<commit_message>
ajustes no jmendes e inicio do desenvolvimento do belgo
</commit_message>
<xml_diff>
--- a/src/bots/jmendes/excel_files/Robô Jmendes.xlsx
+++ b/src/bots/jmendes/excel_files/Robô Jmendes.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29704"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="67292" documentId="11_92485C45C1F39E42E268565A893E8C18510380CC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78C9ACE8-3DD9-4B8D-BE69-AFF4575C07A7}"/>
+  <xr:revisionPtr revIDLastSave="67344" documentId="11_92485C45C1F39E42E268565A893E8C18510380CC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4975D155-B1FA-46BF-A2EE-4381538FE229}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="391">
   <si>
     <t>Data</t>
   </si>
@@ -85,94 +85,94 @@
     <t>Situação Final</t>
   </si>
   <si>
-    <t>KRR7D11</t>
-  </si>
-  <si>
-    <t>Joel Martins dos Santos</t>
+    <t>NJZ0571</t>
+  </si>
+  <si>
+    <t>Edinaldo Rodrigo De Almeida</t>
+  </si>
+  <si>
+    <t>Levolog</t>
+  </si>
+  <si>
+    <t>08579947000291</t>
+  </si>
+  <si>
+    <t>08689024000292</t>
+  </si>
+  <si>
+    <t>JMN</t>
+  </si>
+  <si>
+    <t>VSB</t>
+  </si>
+  <si>
+    <t>Scoff</t>
+  </si>
+  <si>
+    <t>Patrag</t>
+  </si>
+  <si>
+    <t>Desterro de Entre Rios x Jeceaba</t>
+  </si>
+  <si>
+    <t>Piracema x Jeceaba</t>
+  </si>
+  <si>
+    <t>Piracema x Ouro Preto</t>
+  </si>
+  <si>
+    <t>Tarifa</t>
+  </si>
+  <si>
+    <t>08579947000372</t>
+  </si>
+  <si>
+    <t>Destinatário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">08689024000292 </t>
+  </si>
+  <si>
+    <t>33592510043040</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ferro + </t>
+  </si>
+  <si>
+    <t>21256870000287</t>
+  </si>
+  <si>
+    <t>05869287000295</t>
+  </si>
+  <si>
+    <t>Tipo Proprietario</t>
+  </si>
+  <si>
+    <t>Hedilermano Neves</t>
+  </si>
+  <si>
+    <t>HFD4C57</t>
+  </si>
+  <si>
+    <t>Rafael De Andrade</t>
+  </si>
+  <si>
+    <t>OUU8E02</t>
+  </si>
+  <si>
+    <t>Nivaldo Rosario Teixiera Alves Junior</t>
+  </si>
+  <si>
+    <t>OPR1D91</t>
+  </si>
+  <si>
+    <t>Weliton Cardoso Dos Santos</t>
+  </si>
+  <si>
+    <t>QNQ5F49</t>
   </si>
   <si>
     <t xml:space="preserve">FRETO LOG </t>
-  </si>
-  <si>
-    <t>08579947000291</t>
-  </si>
-  <si>
-    <t>08689024000292</t>
-  </si>
-  <si>
-    <t>JMN</t>
-  </si>
-  <si>
-    <t>VSB</t>
-  </si>
-  <si>
-    <t>Scoff</t>
-  </si>
-  <si>
-    <t>Patrag</t>
-  </si>
-  <si>
-    <t>Desterro de Entre Rios x Jeceaba</t>
-  </si>
-  <si>
-    <t>Piracema x Jeceaba</t>
-  </si>
-  <si>
-    <t>Piracema x Ouro Preto</t>
-  </si>
-  <si>
-    <t>Tarifa</t>
-  </si>
-  <si>
-    <t>08579947000372</t>
-  </si>
-  <si>
-    <t>Destinatário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">08689024000292 </t>
-  </si>
-  <si>
-    <t>33592510043040</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ferro + </t>
-  </si>
-  <si>
-    <t>21256870000287</t>
-  </si>
-  <si>
-    <t>05869287000295</t>
-  </si>
-  <si>
-    <t>Tipo Proprietario</t>
-  </si>
-  <si>
-    <t>Hedilermano Neves</t>
-  </si>
-  <si>
-    <t>HFD4C57</t>
-  </si>
-  <si>
-    <t>Levolog</t>
-  </si>
-  <si>
-    <t>Rafael De Andrade</t>
-  </si>
-  <si>
-    <t>OUU8E02</t>
-  </si>
-  <si>
-    <t>Nivaldo Rosario Teixiera Alves Junior</t>
-  </si>
-  <si>
-    <t>OPR1D91</t>
-  </si>
-  <si>
-    <t>Weliton Cardoso Dos Santos</t>
-  </si>
-  <si>
-    <t>QNQ5F49</t>
   </si>
   <si>
     <t>Anderson David Reis</t>
@@ -962,12 +962,6 @@
     <t>HIM3822</t>
   </si>
   <si>
-    <t>Edinaldo Rodrigo De Almeida</t>
-  </si>
-  <si>
-    <t>NJZ0571</t>
-  </si>
-  <si>
     <t>Rodrigo de Oliveira</t>
   </si>
   <si>
@@ -1119,6 +1113,9 @@
   </si>
   <si>
     <t>JOEL MARTINS DOS SANTOS</t>
+  </si>
+  <si>
+    <t>KRR7D11</t>
   </si>
   <si>
     <t>MATHEUS FELIPE DIAS</t>
@@ -2252,13 +2249,13 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" s="62">
-        <v>46029</v>
+        <v>46030</v>
       </c>
       <c r="B2" s="1">
-        <v>635988</v>
+        <v>635496</v>
       </c>
       <c r="C2" s="1">
-        <v>757316229</v>
+        <v>756133740</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>15</v>
@@ -2270,13 +2267,13 @@
         <v>17</v>
       </c>
       <c r="G2" s="1">
-        <v>26360</v>
+        <v>25950</v>
       </c>
       <c r="H2" s="59">
         <v>97</v>
       </c>
       <c r="I2" s="59">
-        <v>1989</v>
+        <v>2797</v>
       </c>
       <c r="J2" s="59">
         <v>22666</v>
@@ -3006,49 +3003,49 @@
         <v>37</v>
       </c>
       <c r="D2" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.75">
       <c r="A3" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B3" s="23">
         <v>756250122</v>
       </c>
       <c r="C3" s="26" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D3" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.75">
       <c r="A4" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B4" s="23">
         <v>746942722</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D4" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.75">
       <c r="A5" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B5" s="23">
         <v>746945612</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D5" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.75">
@@ -3062,7 +3059,7 @@
         <v>46</v>
       </c>
       <c r="D6" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.75">
@@ -3076,7 +3073,7 @@
         <v>48</v>
       </c>
       <c r="D7" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.75">
@@ -3090,7 +3087,7 @@
         <v>50</v>
       </c>
       <c r="D8" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.75">
@@ -3104,7 +3101,7 @@
         <v>52</v>
       </c>
       <c r="D9" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15.75">
@@ -3118,7 +3115,7 @@
         <v>54</v>
       </c>
       <c r="D10" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15.75">
@@ -3132,7 +3129,7 @@
         <v>56</v>
       </c>
       <c r="D11" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15.75">
@@ -3146,7 +3143,7 @@
         <v>58</v>
       </c>
       <c r="D12" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="15.75">
@@ -3158,7 +3155,7 @@
         <v>60</v>
       </c>
       <c r="D13" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="15.75">
@@ -3172,7 +3169,7 @@
         <v>62</v>
       </c>
       <c r="D14" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="15.75">
@@ -3186,7 +3183,7 @@
         <v>64</v>
       </c>
       <c r="D15" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="15.75">
@@ -3200,7 +3197,7 @@
         <v>66</v>
       </c>
       <c r="D16" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15.75">
@@ -3214,7 +3211,7 @@
         <v>68</v>
       </c>
       <c r="D17" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="15.75">
@@ -3228,7 +3225,7 @@
         <v>70</v>
       </c>
       <c r="D18" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="15.75">
@@ -3242,7 +3239,7 @@
         <v>72</v>
       </c>
       <c r="D19" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="15.75">
@@ -3256,7 +3253,7 @@
         <v>74</v>
       </c>
       <c r="D20" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="15.75">
@@ -3270,7 +3267,7 @@
         <v>76</v>
       </c>
       <c r="D21" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="15.75">
@@ -3284,7 +3281,7 @@
         <v>78</v>
       </c>
       <c r="D22" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="15.75">
@@ -3298,7 +3295,7 @@
         <v>80</v>
       </c>
       <c r="D23" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="15.75">
@@ -3310,7 +3307,7 @@
       </c>
       <c r="C24" s="26"/>
       <c r="D24" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="15.75">
@@ -3334,7 +3331,7 @@
         <v>84</v>
       </c>
       <c r="D26" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="15.75">
@@ -3348,7 +3345,7 @@
         <v>86</v>
       </c>
       <c r="D27" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="15.75">
@@ -3362,7 +3359,7 @@
         <v>88</v>
       </c>
       <c r="D28" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="15.75">
@@ -3376,7 +3373,7 @@
         <v>90</v>
       </c>
       <c r="D29" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="15.75">
@@ -3390,7 +3387,7 @@
         <v>92</v>
       </c>
       <c r="D30" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -3404,7 +3401,7 @@
         <v>94</v>
       </c>
       <c r="D31" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="15.75">
@@ -3418,7 +3415,7 @@
         <v>96</v>
       </c>
       <c r="D32" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="15.75">
@@ -3432,7 +3429,7 @@
         <v>98</v>
       </c>
       <c r="D33" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="15.75">
@@ -3446,7 +3443,7 @@
         <v>100</v>
       </c>
       <c r="D34" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="15.75">
@@ -3460,7 +3457,7 @@
         <v>102</v>
       </c>
       <c r="D35" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="15.75">
@@ -3474,7 +3471,7 @@
         <v>104</v>
       </c>
       <c r="D36" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="15.75">
@@ -3488,7 +3485,7 @@
         <v>106</v>
       </c>
       <c r="D37" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="15.75">
@@ -3502,7 +3499,7 @@
         <v>108</v>
       </c>
       <c r="D38" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="15.75">
@@ -3516,7 +3513,7 @@
         <v>110</v>
       </c>
       <c r="D39" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="15.75">
@@ -3530,7 +3527,7 @@
         <v>112</v>
       </c>
       <c r="D40" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="15.75">
@@ -3544,7 +3541,7 @@
         <v>114</v>
       </c>
       <c r="D41" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="15.75">
@@ -3558,7 +3555,7 @@
         <v>116</v>
       </c>
       <c r="D42" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="15.75">
@@ -3572,7 +3569,7 @@
         <v>117</v>
       </c>
       <c r="D43" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="15.75">
@@ -3586,7 +3583,7 @@
         <v>119</v>
       </c>
       <c r="D44" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="15.75">
@@ -3600,7 +3597,7 @@
         <v>121</v>
       </c>
       <c r="D45" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="15.75">
@@ -3614,7 +3611,7 @@
         <v>123</v>
       </c>
       <c r="D46" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="15.75">
@@ -3628,7 +3625,7 @@
         <v>125</v>
       </c>
       <c r="D47" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="15.75">
@@ -3642,7 +3639,7 @@
         <v>127</v>
       </c>
       <c r="D48" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="15.75">
@@ -3656,7 +3653,7 @@
         <v>129</v>
       </c>
       <c r="D49" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="15.75">
@@ -3670,7 +3667,7 @@
         <v>131</v>
       </c>
       <c r="D50" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="15.75">
@@ -3684,7 +3681,7 @@
         <v>133</v>
       </c>
       <c r="D51" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="15.75">
@@ -3698,7 +3695,7 @@
         <v>135</v>
       </c>
       <c r="D52" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="15.75">
@@ -3712,7 +3709,7 @@
         <v>137</v>
       </c>
       <c r="D53" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="E53" s="46" t="s">
         <v>138</v>
@@ -3729,7 +3726,7 @@
         <v>140</v>
       </c>
       <c r="D54" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="15.75">
@@ -3743,7 +3740,7 @@
         <v>142</v>
       </c>
       <c r="D55" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="15.75">
@@ -3757,7 +3754,7 @@
         <v>144</v>
       </c>
       <c r="D56" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="15.75">
@@ -3771,7 +3768,7 @@
         <v>146</v>
       </c>
       <c r="D57" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="15.75">
@@ -3783,7 +3780,7 @@
         <v>148</v>
       </c>
       <c r="D58" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="15.75">
@@ -3797,7 +3794,7 @@
         <v>150</v>
       </c>
       <c r="D59" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="15.75">
@@ -3809,7 +3806,7 @@
         <v>152</v>
       </c>
       <c r="D60" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="15.75">
@@ -3823,7 +3820,7 @@
         <v>154</v>
       </c>
       <c r="D61" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="15.75">
@@ -3837,7 +3834,7 @@
         <v>156</v>
       </c>
       <c r="D62" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="15.75">
@@ -3851,7 +3848,7 @@
         <v>158</v>
       </c>
       <c r="D63" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="15.75">
@@ -3865,7 +3862,7 @@
         <v>160</v>
       </c>
       <c r="D64" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="15.75" customHeight="1">
@@ -3879,7 +3876,7 @@
         <v>162</v>
       </c>
       <c r="D65" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="15.75">
@@ -3893,7 +3890,7 @@
         <v>164</v>
       </c>
       <c r="D66" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="15.75">
@@ -3907,7 +3904,7 @@
         <v>166</v>
       </c>
       <c r="D67" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="15.75">
@@ -3921,7 +3918,7 @@
         <v>108</v>
       </c>
       <c r="D68" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="15.75">
@@ -3935,7 +3932,7 @@
         <v>169</v>
       </c>
       <c r="D69" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="15.75">
@@ -3949,7 +3946,7 @@
         <v>171</v>
       </c>
       <c r="D70" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="15.75">
@@ -3963,7 +3960,7 @@
         <v>173</v>
       </c>
       <c r="D71" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="15.75">
@@ -3977,7 +3974,7 @@
         <v>176</v>
       </c>
       <c r="D72" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="15.75">
@@ -3991,7 +3988,7 @@
         <v>178</v>
       </c>
       <c r="D73" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="E73" s="46" t="s">
         <v>138</v>
@@ -4008,7 +4005,7 @@
         <v>180</v>
       </c>
       <c r="D74" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="15.75">
@@ -4022,7 +4019,7 @@
         <v>121</v>
       </c>
       <c r="D75" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="15.75">
@@ -4036,7 +4033,7 @@
         <v>183</v>
       </c>
       <c r="D76" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="15.75">
@@ -4050,7 +4047,7 @@
         <v>185</v>
       </c>
       <c r="D77" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="15.75">
@@ -4064,7 +4061,7 @@
         <v>187</v>
       </c>
       <c r="D78" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="79" spans="1:5" ht="15.75">
@@ -4078,7 +4075,7 @@
         <v>86</v>
       </c>
       <c r="D79" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="80" spans="1:5" ht="15.75">
@@ -4092,7 +4089,7 @@
         <v>190</v>
       </c>
       <c r="D80" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="81" spans="1:4" ht="15.75">
@@ -4106,7 +4103,7 @@
         <v>191</v>
       </c>
       <c r="D81" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="82" spans="1:4" ht="15.75">
@@ -4120,7 +4117,7 @@
         <v>193</v>
       </c>
       <c r="D82" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="83" spans="1:4" ht="15.75">
@@ -4134,7 +4131,7 @@
         <v>195</v>
       </c>
       <c r="D83" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="84" spans="1:4" ht="15.75">
@@ -4148,7 +4145,7 @@
         <v>197</v>
       </c>
       <c r="D84" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="85" spans="1:4" ht="15.75">
@@ -4160,7 +4157,7 @@
       </c>
       <c r="C85" s="29"/>
       <c r="D85" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="86" spans="1:4" ht="15.75">
@@ -4174,7 +4171,7 @@
         <v>200</v>
       </c>
       <c r="D86" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="87" spans="1:4" ht="15.75">
@@ -4188,7 +4185,7 @@
         <v>84</v>
       </c>
       <c r="D87" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="88" spans="1:4" ht="15.75">
@@ -4202,7 +4199,7 @@
         <v>203</v>
       </c>
       <c r="D88" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="89" spans="1:4" ht="15.75">
@@ -4216,7 +4213,7 @@
         <v>205</v>
       </c>
       <c r="D89" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="90" spans="1:4" ht="15.75">
@@ -4230,7 +4227,7 @@
         <v>207</v>
       </c>
       <c r="D90" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="91" spans="1:4" ht="15.75">
@@ -4244,7 +4241,7 @@
         <v>209</v>
       </c>
       <c r="D91" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="15.75">
@@ -4258,7 +4255,7 @@
         <v>211</v>
       </c>
       <c r="D92" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="93" spans="1:4" ht="15.75">
@@ -4272,7 +4269,7 @@
         <v>212</v>
       </c>
       <c r="D93" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="94" spans="1:4" ht="15.75">
@@ -4286,7 +4283,7 @@
         <v>214</v>
       </c>
       <c r="D94" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="95" spans="1:4" ht="15.75">
@@ -4300,7 +4297,7 @@
         <v>216</v>
       </c>
       <c r="D95" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="96" spans="1:4" ht="15.75">
@@ -4314,7 +4311,7 @@
         <v>218</v>
       </c>
       <c r="D96" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="97" spans="1:4" ht="15.75">
@@ -4328,7 +4325,7 @@
         <v>220</v>
       </c>
       <c r="D97" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="98" spans="1:4" ht="15.75">
@@ -4342,7 +4339,7 @@
         <v>222</v>
       </c>
       <c r="D98" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="99" spans="1:4" ht="15.75">
@@ -4356,7 +4353,7 @@
         <v>224</v>
       </c>
       <c r="D99" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="100" spans="1:4" ht="15.75">
@@ -4370,7 +4367,7 @@
         <v>226</v>
       </c>
       <c r="D100" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="101" spans="1:4" ht="15.75">
@@ -4384,7 +4381,7 @@
         <v>228</v>
       </c>
       <c r="D101" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="102" spans="1:4" ht="15.75">
@@ -4398,7 +4395,7 @@
         <v>230</v>
       </c>
       <c r="D102" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="103" spans="1:4" ht="15.75">
@@ -4412,7 +4409,7 @@
         <v>232</v>
       </c>
       <c r="D103" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="104" spans="1:4" ht="15.75">
@@ -4423,10 +4420,10 @@
         <v>755660156</v>
       </c>
       <c r="C104" s="29" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D104" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="105" spans="1:4">
@@ -4438,7 +4435,7 @@
         <v>90</v>
       </c>
       <c r="D105" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="106" spans="1:4" ht="15.75">
@@ -4452,7 +4449,7 @@
         <v>235</v>
       </c>
       <c r="D106" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="107" spans="1:4" ht="15.75">
@@ -4466,7 +4463,7 @@
         <v>237</v>
       </c>
       <c r="D107" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="108" spans="1:4" ht="15.75">
@@ -4480,7 +4477,7 @@
         <v>239</v>
       </c>
       <c r="D108" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="109" spans="1:4" ht="15.75">
@@ -4494,7 +4491,7 @@
         <v>241</v>
       </c>
       <c r="D109" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="110" spans="1:4" ht="15.75">
@@ -4508,7 +4505,7 @@
         <v>243</v>
       </c>
       <c r="D110" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="111" spans="1:4" ht="15.75">
@@ -4522,7 +4519,7 @@
         <v>245</v>
       </c>
       <c r="D111" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="112" spans="1:4" ht="15.75">
@@ -4536,7 +4533,7 @@
         <v>247</v>
       </c>
       <c r="D112" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="113" spans="1:4" ht="15.75">
@@ -4550,7 +4547,7 @@
         <v>249</v>
       </c>
       <c r="D113" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="114" spans="1:4" ht="15.75">
@@ -4564,7 +4561,7 @@
         <v>251</v>
       </c>
       <c r="D114" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="115" spans="1:4" ht="15.75">
@@ -4578,7 +4575,7 @@
         <v>253</v>
       </c>
       <c r="D115" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="116" spans="1:4" ht="15.75">
@@ -4592,7 +4589,7 @@
         <v>255</v>
       </c>
       <c r="D116" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="117" spans="1:4" ht="15.75">
@@ -4606,7 +4603,7 @@
         <v>257</v>
       </c>
       <c r="D117" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="118" spans="1:4" ht="15.75">
@@ -4620,7 +4617,7 @@
         <v>259</v>
       </c>
       <c r="D118" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="119" spans="1:4" ht="15.75">
@@ -4634,7 +4631,7 @@
         <v>261</v>
       </c>
       <c r="D119" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="120" spans="1:4" ht="15.75">
@@ -4648,7 +4645,7 @@
         <v>263</v>
       </c>
       <c r="D120" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="121" spans="1:4" ht="15.75">
@@ -4662,7 +4659,7 @@
         <v>265</v>
       </c>
       <c r="D121" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="122" spans="1:4" ht="15.75">
@@ -4676,7 +4673,7 @@
         <v>267</v>
       </c>
       <c r="D122" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="123" spans="1:4" ht="15.75">
@@ -4690,7 +4687,7 @@
         <v>269</v>
       </c>
       <c r="D123" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="124" spans="1:4" ht="15.75">
@@ -4704,7 +4701,7 @@
         <v>271</v>
       </c>
       <c r="D124" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="125" spans="1:4" ht="15.75">
@@ -4718,7 +4715,7 @@
         <v>273</v>
       </c>
       <c r="D125" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="126" spans="1:4" ht="15.75">
@@ -4744,7 +4741,7 @@
         <v>277</v>
       </c>
       <c r="D127" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="128" spans="1:4" ht="15.75">
@@ -4758,7 +4755,7 @@
         <v>257</v>
       </c>
       <c r="D128" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="129" spans="1:4" ht="15.75">
@@ -4772,7 +4769,7 @@
         <v>280</v>
       </c>
       <c r="D129" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="130" spans="1:4" ht="15.75">
@@ -4786,7 +4783,7 @@
         <v>282</v>
       </c>
       <c r="D130" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="131" spans="1:4" ht="15.75">
@@ -4800,7 +4797,7 @@
         <v>284</v>
       </c>
       <c r="D131" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="132" spans="1:4" ht="15.75">
@@ -4814,7 +4811,7 @@
         <v>286</v>
       </c>
       <c r="D132" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="133" spans="1:4" ht="15.75">
@@ -4828,7 +4825,7 @@
         <v>288</v>
       </c>
       <c r="D133" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="134" spans="1:4" ht="15.75">
@@ -4840,7 +4837,7 @@
         <v>290</v>
       </c>
       <c r="D134" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="135" spans="1:4" ht="15.75">
@@ -4854,7 +4851,7 @@
         <v>292</v>
       </c>
       <c r="D135" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="136" spans="1:4" ht="15.75">
@@ -4868,7 +4865,7 @@
         <v>294</v>
       </c>
       <c r="D136" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="137" spans="1:4" ht="15.75">
@@ -4882,7 +4879,7 @@
         <v>296</v>
       </c>
       <c r="D137" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="138" spans="1:4" ht="15.75">
@@ -4896,7 +4893,7 @@
         <v>298</v>
       </c>
       <c r="D138" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="139" spans="1:4" ht="15.75">
@@ -4922,7 +4919,7 @@
         <v>302</v>
       </c>
       <c r="D140" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="141" spans="1:4" ht="15.75">
@@ -4936,7 +4933,7 @@
         <v>304</v>
       </c>
       <c r="D141" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="142" spans="1:4" ht="15.75">
@@ -4950,26 +4947,26 @@
         <v>306</v>
       </c>
       <c r="D142" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="143" spans="1:4" ht="15.75">
       <c r="A143" s="5" t="s">
-        <v>307</v>
+        <v>16</v>
       </c>
       <c r="B143" s="7">
         <v>756133740</v>
       </c>
       <c r="C143" s="29" t="s">
-        <v>308</v>
+        <v>15</v>
       </c>
       <c r="D143" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="144" spans="1:4" ht="15.75">
       <c r="A144" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="B144" s="7">
         <v>752390336</v>
@@ -4978,220 +4975,220 @@
         <v>98</v>
       </c>
       <c r="D144" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="145" spans="1:4" ht="15.75">
       <c r="A145" s="5" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B145" s="7">
         <v>748663853</v>
       </c>
       <c r="C145" s="29" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="D145" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="146" spans="1:4" ht="15.75">
       <c r="A146" s="5" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B146" s="7">
         <v>757522479</v>
       </c>
       <c r="C146" s="29" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="D146" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="147" spans="1:4" ht="15.75">
       <c r="A147" s="5" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="B147" s="7">
         <v>748663887</v>
       </c>
       <c r="C147" s="29" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="D147" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="148" spans="1:4" ht="15.75">
       <c r="A148" s="5" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B148" s="7">
         <v>752390401</v>
       </c>
       <c r="C148" s="29" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D148" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="149" spans="1:4" ht="15.75">
       <c r="A149" s="5" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="B149" s="7">
         <v>754842326</v>
       </c>
       <c r="C149" s="29" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="D149" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="150" spans="1:4" ht="15.75">
       <c r="A150" s="5" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B150" s="7">
         <v>748173762</v>
       </c>
       <c r="C150" s="29" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D150" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="151" spans="1:4" ht="15.75">
       <c r="A151" s="5" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B151" s="7">
         <v>752390252</v>
       </c>
       <c r="C151" s="29" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D151" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="152" spans="1:4" ht="15.75">
       <c r="A152" s="5" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="B152" s="7">
         <v>752390260</v>
       </c>
       <c r="C152" s="29" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D152" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="153" spans="1:4" ht="15.75">
       <c r="A153" s="5" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="B153" s="7">
         <v>748663754</v>
       </c>
       <c r="C153" s="29" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D153" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="154" spans="1:4" ht="15.75">
       <c r="A154" s="5" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="B154" s="7">
         <v>754842334</v>
       </c>
       <c r="C154" s="29" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D154" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="155" spans="1:4" ht="15.75">
       <c r="A155" s="5" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="B155" s="7">
         <v>748663663</v>
       </c>
       <c r="C155" s="29" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="D155" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="156" spans="1:4" ht="15.75">
       <c r="A156" s="5" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="B156" s="7">
         <v>754845089</v>
       </c>
       <c r="C156" s="29" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="D156" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="157" spans="1:4" ht="15.75">
       <c r="A157" s="5" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B157" s="7">
         <v>754803260</v>
       </c>
       <c r="C157" s="29" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="D157" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="158" spans="1:4" ht="15.75">
       <c r="A158" s="5" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="B158" s="7">
         <v>748663432</v>
       </c>
       <c r="C158" s="29" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="D158" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="159" spans="1:4" ht="15.75">
       <c r="A159" s="5" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B159" s="7">
         <v>754845055</v>
       </c>
       <c r="C159" s="29"/>
       <c r="D159" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="160" spans="1:4" ht="15.75">
       <c r="A160" s="5" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B160" s="7">
         <v>754845147</v>
@@ -5200,21 +5197,21 @@
         <v>52</v>
       </c>
       <c r="D160" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="161" spans="1:4" ht="15.75">
       <c r="A161" s="5" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="B161" s="7">
         <v>754842342</v>
       </c>
       <c r="C161" s="29" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="D161" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="162" spans="1:4" ht="15.75">
@@ -5228,54 +5225,54 @@
         <v>166</v>
       </c>
       <c r="D162" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="163" spans="1:4" ht="15.75">
       <c r="A163" s="5" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="B163" s="7">
         <v>757316278</v>
       </c>
       <c r="C163" s="29" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D163" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="164" spans="1:4" ht="15.75">
       <c r="A164" s="5" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="B164" s="7">
         <v>755660149</v>
       </c>
       <c r="C164" s="29" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D164" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="165" spans="1:4" ht="15.75">
       <c r="A165" s="5" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B165" s="7">
         <v>756250114</v>
       </c>
       <c r="C165" s="29" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="D165" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="166" spans="1:4" ht="15.75">
       <c r="A166" s="5" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B166" s="7">
         <v>756250148</v>
@@ -5284,40 +5281,40 @@
         <v>205</v>
       </c>
       <c r="D166" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="167" spans="1:4" ht="15.75">
       <c r="A167" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B167" s="7">
         <v>756249959</v>
       </c>
       <c r="C167" s="29" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D167" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="168" spans="1:4" ht="15.75">
       <c r="A168" s="5" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="B168" s="7">
         <v>756249967</v>
       </c>
       <c r="C168" s="29" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="D168" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="169" spans="1:4" ht="15.75">
       <c r="A169" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B169" s="7">
         <v>756250437</v>
@@ -5326,26 +5323,26 @@
         <v>228</v>
       </c>
       <c r="D169" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="170" spans="1:4" ht="15.75">
       <c r="A170" s="5" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B170" s="7">
         <v>756250445</v>
       </c>
       <c r="C170" s="29" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="D170" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="171" spans="1:4" ht="15.75">
       <c r="A171" s="5" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="B171" s="7">
         <v>756250304</v>
@@ -5354,91 +5351,91 @@
         <v>54</v>
       </c>
       <c r="D171" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="172" spans="1:4" ht="15.75">
       <c r="A172" s="5" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B172" s="7">
         <v>757025119</v>
       </c>
       <c r="C172" s="29" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="D172" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="173" spans="1:4" ht="15.75">
       <c r="A173" s="5" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="B173" s="7">
         <v>757025176</v>
       </c>
       <c r="C173" s="29" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="D173" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="174" spans="1:4" ht="15.75">
       <c r="A174" s="5" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B174" s="7">
         <v>757316229</v>
       </c>
       <c r="C174" s="29" t="s">
-        <v>15</v>
+        <v>358</v>
       </c>
       <c r="D174" s="32" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="175" spans="1:4" ht="15.75">
       <c r="A175" s="5" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B175" s="7">
         <v>757316245</v>
       </c>
       <c r="C175" s="29" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="D175" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="176" spans="1:4" ht="15.75">
       <c r="A176" s="5" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B176" s="7">
         <v>757522487</v>
       </c>
       <c r="C176" s="29" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D176" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="177" spans="1:4" ht="15.75">
       <c r="A177" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B177" s="7">
         <v>757316286</v>
       </c>
       <c r="C177" s="29" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D177" s="32" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
     </row>
     <row r="178" spans="1:4" ht="15.75">
@@ -5531,7 +5528,7 @@
   <sheetData>
     <row r="2" spans="1:13">
       <c r="A2" s="42" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="B2" s="35"/>
       <c r="C2" s="35"/>
@@ -5540,7 +5537,7 @@
       <c r="F2" s="35"/>
       <c r="G2" s="35"/>
       <c r="H2" s="51" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="I2" s="52"/>
       <c r="J2" s="52"/>
@@ -5555,40 +5552,40 @@
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="37" t="s">
+        <v>366</v>
+      </c>
+      <c r="B4" s="33" t="s">
         <v>367</v>
       </c>
-      <c r="B4" s="33" t="s">
+      <c r="C4" s="33" t="s">
         <v>368</v>
       </c>
-      <c r="C4" s="33" t="s">
+      <c r="D4" s="33" t="s">
         <v>369</v>
       </c>
-      <c r="D4" s="33" t="s">
+      <c r="E4" s="33" t="s">
         <v>370</v>
       </c>
-      <c r="E4" s="33" t="s">
+      <c r="G4" s="33" t="s">
         <v>371</v>
       </c>
-      <c r="G4" s="33" t="s">
+      <c r="H4" s="37" t="s">
+        <v>366</v>
+      </c>
+      <c r="I4" s="33" t="s">
+        <v>367</v>
+      </c>
+      <c r="J4" s="33" t="s">
+        <v>368</v>
+      </c>
+      <c r="K4" s="33" t="s">
+        <v>369</v>
+      </c>
+      <c r="L4" s="33" t="s">
+        <v>370</v>
+      </c>
+      <c r="M4" s="58" t="s">
         <v>372</v>
-      </c>
-      <c r="H4" s="37" t="s">
-        <v>367</v>
-      </c>
-      <c r="I4" s="33" t="s">
-        <v>368</v>
-      </c>
-      <c r="J4" s="33" t="s">
-        <v>369</v>
-      </c>
-      <c r="K4" s="33" t="s">
-        <v>370</v>
-      </c>
-      <c r="L4" s="33" t="s">
-        <v>371</v>
-      </c>
-      <c r="M4" s="58" t="s">
-        <v>373</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -5598,40 +5595,40 @@
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="31" t="s">
+        <v>373</v>
+      </c>
+      <c r="B6" s="32" t="s">
+        <v>373</v>
+      </c>
+      <c r="C6" s="32" t="s">
+        <v>373</v>
+      </c>
+      <c r="D6" s="50" t="s">
         <v>374</v>
       </c>
-      <c r="B6" s="32" t="s">
-        <v>374</v>
-      </c>
-      <c r="C6" s="32" t="s">
-        <v>374</v>
-      </c>
-      <c r="D6" s="50" t="s">
+      <c r="E6" s="32" t="s">
+        <v>373</v>
+      </c>
+      <c r="G6" s="32" t="s">
+        <v>373</v>
+      </c>
+      <c r="H6" s="31" t="s">
+        <v>373</v>
+      </c>
+      <c r="I6" s="32" t="s">
+        <v>373</v>
+      </c>
+      <c r="J6" s="32" t="s">
+        <v>373</v>
+      </c>
+      <c r="K6" s="50" t="s">
         <v>375</v>
       </c>
-      <c r="E6" s="32" t="s">
-        <v>374</v>
-      </c>
-      <c r="G6" s="32" t="s">
-        <v>374</v>
-      </c>
-      <c r="H6" s="31" t="s">
-        <v>374</v>
-      </c>
-      <c r="I6" s="32" t="s">
-        <v>374</v>
-      </c>
-      <c r="J6" s="32" t="s">
-        <v>374</v>
-      </c>
-      <c r="K6" s="50" t="s">
-        <v>376</v>
-      </c>
       <c r="L6" s="32" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="M6" s="36" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -5641,41 +5638,41 @@
     </row>
     <row r="8" spans="1:13" ht="15.75">
       <c r="A8" s="43" t="s">
+        <v>376</v>
+      </c>
+      <c r="B8" s="44" t="s">
         <v>377</v>
       </c>
-      <c r="B8" s="44" t="s">
+      <c r="C8" s="44" t="s">
         <v>378</v>
       </c>
-      <c r="C8" s="44" t="s">
+      <c r="D8" s="44" t="s">
+        <v>378</v>
+      </c>
+      <c r="E8" s="44" t="s">
         <v>379</v>
-      </c>
-      <c r="D8" s="44" t="s">
-        <v>379</v>
-      </c>
-      <c r="E8" s="44" t="s">
-        <v>380</v>
       </c>
       <c r="F8" s="44"/>
       <c r="G8" s="44" t="s">
+        <v>380</v>
+      </c>
+      <c r="H8" s="43" t="s">
         <v>381</v>
       </c>
-      <c r="H8" s="43" t="s">
+      <c r="I8" s="44" t="s">
         <v>382</v>
       </c>
-      <c r="I8" s="44" t="s">
+      <c r="J8" s="44" t="s">
         <v>383</v>
       </c>
-      <c r="J8" s="44" t="s">
+      <c r="K8" s="44" t="s">
+        <v>383</v>
+      </c>
+      <c r="L8" s="44" t="s">
         <v>384</v>
       </c>
-      <c r="K8" s="44" t="s">
-        <v>384</v>
-      </c>
-      <c r="L8" s="44" t="s">
+      <c r="M8" s="44" t="s">
         <v>385</v>
-      </c>
-      <c r="M8" s="44" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -5685,40 +5682,40 @@
     </row>
     <row r="10" spans="1:13">
       <c r="A10" s="31" t="s">
+        <v>386</v>
+      </c>
+      <c r="B10" s="32" t="s">
         <v>387</v>
       </c>
-      <c r="B10" s="32" t="s">
-        <v>388</v>
-      </c>
       <c r="C10" s="32" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D10" s="32" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="G10" s="32" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="H10" s="31" t="s">
+        <v>386</v>
+      </c>
+      <c r="I10" s="32" t="s">
         <v>387</v>
       </c>
-      <c r="I10" s="32" t="s">
-        <v>388</v>
-      </c>
       <c r="J10" s="32" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="K10" s="32" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="L10" s="32" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="M10" s="36" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -5728,40 +5725,40 @@
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="31" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B12" s="32" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C12" s="32" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="D12" s="32" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="G12" s="32" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H12" s="31" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="I12" s="32" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="J12" s="32" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="K12" s="32" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="L12" s="32" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="M12" s="36" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -5771,40 +5768,40 @@
     </row>
     <row r="14" spans="1:13">
       <c r="A14" s="31" t="s">
+        <v>389</v>
+      </c>
+      <c r="B14" s="32" t="s">
         <v>390</v>
       </c>
-      <c r="B14" s="32" t="s">
-        <v>391</v>
-      </c>
       <c r="C14" s="32" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="D14" s="32" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E14" s="32" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="G14" s="32" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="H14" s="31" t="s">
+        <v>389</v>
+      </c>
+      <c r="I14" s="32" t="s">
         <v>390</v>
       </c>
-      <c r="I14" s="32" t="s">
-        <v>391</v>
-      </c>
       <c r="J14" s="32" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="K14" s="32" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="L14" s="32" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="M14" s="36" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -5847,7 +5844,7 @@
     </row>
     <row r="19" spans="1:13">
       <c r="A19" s="50" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="I19" s="34"/>
       <c r="J19" s="54"/>
@@ -5855,7 +5852,7 @@
     </row>
     <row r="20" spans="1:13">
       <c r="A20" s="50" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="I20" s="34"/>
       <c r="J20" s="54"/>

</xml_diff>

<commit_message>
ajustes no worker do jmn e no publisher do belgo
</commit_message>
<xml_diff>
--- a/src/bots/jmendes/excel_files/Robô Jmendes.xlsx
+++ b/src/bots/jmendes/excel_files/Robô Jmendes.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29704"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29711"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="67344" documentId="11_92485C45C1F39E42E268565A893E8C18510380CC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4975D155-B1FA-46BF-A2EE-4381538FE229}"/>
+  <xr:revisionPtr revIDLastSave="67390" documentId="11_92485C45C1F39E42E268565A893E8C18510380CC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B456695-5CB7-49D7-AB3C-53AA9C5A9A68}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -85,10 +85,10 @@
     <t>Situação Final</t>
   </si>
   <si>
-    <t>NJZ0571</t>
-  </si>
-  <si>
-    <t>Edinaldo Rodrigo De Almeida</t>
+    <t>MQN5475</t>
+  </si>
+  <si>
+    <t>Antonio Dos Santos</t>
   </si>
   <si>
     <t>Levolog</t>
@@ -665,12 +665,6 @@
     <t>RGB6E18</t>
   </si>
   <si>
-    <t>Antonio Dos Santos</t>
-  </si>
-  <si>
-    <t>MQN5475</t>
-  </si>
-  <si>
     <t>Milton Vieira Marciano</t>
   </si>
   <si>
@@ -960,6 +954,12 @@
   </si>
   <si>
     <t>HIM3822</t>
+  </si>
+  <si>
+    <t>Edinaldo Rodrigo De Almeida</t>
+  </si>
+  <si>
+    <t>NJZ0571</t>
   </si>
   <si>
     <t>Rodrigo de Oliveira</t>
@@ -2249,13 +2249,13 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" s="62">
-        <v>46030</v>
+        <v>46035</v>
       </c>
       <c r="B2" s="1">
-        <v>635496</v>
+        <v>637502</v>
       </c>
       <c r="C2" s="1">
-        <v>756133740</v>
+        <v>754842318</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>15</v>
@@ -2267,7 +2267,7 @@
         <v>17</v>
       </c>
       <c r="G2" s="1">
-        <v>25950</v>
+        <v>25200</v>
       </c>
       <c r="H2" s="59">
         <v>97</v>
@@ -4232,13 +4232,13 @@
     </row>
     <row r="91" spans="1:4" ht="15.75">
       <c r="A91" s="5" t="s">
-        <v>208</v>
+        <v>16</v>
       </c>
       <c r="B91" s="7">
         <v>754842318</v>
       </c>
       <c r="C91" s="29" t="s">
-        <v>209</v>
+        <v>15</v>
       </c>
       <c r="D91" s="32" t="s">
         <v>17</v>
@@ -4246,13 +4246,13 @@
     </row>
     <row r="92" spans="1:4" ht="15.75">
       <c r="A92" s="5" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B92" s="7">
         <v>748173697</v>
       </c>
       <c r="C92" s="29" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D92" s="32" t="s">
         <v>17</v>
@@ -4266,7 +4266,7 @@
         <v>746942875</v>
       </c>
       <c r="C93" s="29" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="D93" s="32" t="s">
         <v>44</v>
@@ -4274,13 +4274,13 @@
     </row>
     <row r="94" spans="1:4" ht="15.75">
       <c r="A94" s="5" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B94" s="7">
         <v>748173747</v>
       </c>
       <c r="C94" s="29" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="D94" s="32" t="s">
         <v>44</v>
@@ -4288,13 +4288,13 @@
     </row>
     <row r="95" spans="1:4" ht="15.75">
       <c r="A95" s="5" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B95" s="7">
         <v>748663903</v>
       </c>
       <c r="C95" s="29" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="D95" s="32" t="s">
         <v>44</v>
@@ -4302,13 +4302,13 @@
     </row>
     <row r="96" spans="1:4" ht="15.75">
       <c r="A96" s="5" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B96" s="7">
         <v>748662996</v>
       </c>
       <c r="C96" s="29" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="D96" s="32" t="s">
         <v>44</v>
@@ -4316,13 +4316,13 @@
     </row>
     <row r="97" spans="1:4" ht="15.75">
       <c r="A97" s="5" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B97" s="7">
         <v>748663911</v>
       </c>
       <c r="C97" s="29" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="D97" s="32" t="s">
         <v>44</v>
@@ -4330,13 +4330,13 @@
     </row>
     <row r="98" spans="1:4" ht="15.75">
       <c r="A98" s="5" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B98" s="7">
         <v>748663390</v>
       </c>
       <c r="C98" s="29" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D98" s="32" t="s">
         <v>44</v>
@@ -4344,13 +4344,13 @@
     </row>
     <row r="99" spans="1:4" ht="15.75">
       <c r="A99" s="5" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B99" s="7">
         <v>748663382</v>
       </c>
       <c r="C99" s="29" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="D99" s="32" t="s">
         <v>44</v>
@@ -4358,13 +4358,13 @@
     </row>
     <row r="100" spans="1:4" ht="15.75">
       <c r="A100" s="5" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B100" s="7">
         <v>750635237</v>
       </c>
       <c r="C100" s="29" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D100" s="32" t="s">
         <v>44</v>
@@ -4372,13 +4372,13 @@
     </row>
     <row r="101" spans="1:4" ht="15.75">
       <c r="A101" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B101" s="7">
         <v>748664422</v>
       </c>
       <c r="C101" s="29" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D101" s="32" t="s">
         <v>44</v>
@@ -4386,13 +4386,13 @@
     </row>
     <row r="102" spans="1:4" ht="15.75">
       <c r="A102" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B102" s="7">
         <v>748664430</v>
       </c>
       <c r="C102" s="29" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D102" s="32" t="s">
         <v>44</v>
@@ -4400,13 +4400,13 @@
     </row>
     <row r="103" spans="1:4" ht="15.75">
       <c r="A103" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B103" s="7">
         <v>748664406</v>
       </c>
       <c r="C103" s="29" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D103" s="32" t="s">
         <v>17</v>
@@ -4414,7 +4414,7 @@
     </row>
     <row r="104" spans="1:4" ht="15.75">
       <c r="A104" s="5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B104" s="7">
         <v>755660156</v>
@@ -4428,7 +4428,7 @@
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="5" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B105" s="6"/>
       <c r="C105" s="29" t="s">
@@ -4446,7 +4446,7 @@
         <v>746181107</v>
       </c>
       <c r="C106" s="29" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="D106" s="32" t="s">
         <v>17</v>
@@ -4454,13 +4454,13 @@
     </row>
     <row r="107" spans="1:4" ht="15.75">
       <c r="A107" s="5" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B107" s="7">
         <v>750633877</v>
       </c>
       <c r="C107" s="29" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="D107" s="32" t="s">
         <v>17</v>
@@ -4468,13 +4468,13 @@
     </row>
     <row r="108" spans="1:4" ht="15.75">
       <c r="A108" s="5" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B108" s="7">
         <v>750634263</v>
       </c>
       <c r="C108" s="29" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D108" s="32" t="s">
         <v>17</v>
@@ -4482,13 +4482,13 @@
     </row>
     <row r="109" spans="1:4" ht="15.75">
       <c r="A109" s="5" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B109" s="7">
         <v>748663820</v>
       </c>
       <c r="C109" s="29" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="D109" s="32" t="s">
         <v>44</v>
@@ -4496,13 +4496,13 @@
     </row>
     <row r="110" spans="1:4" ht="15.75">
       <c r="A110" s="5" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B110" s="7">
         <v>748664471</v>
       </c>
       <c r="C110" s="29" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="D110" s="32" t="s">
         <v>17</v>
@@ -4510,13 +4510,13 @@
     </row>
     <row r="111" spans="1:4" ht="15.75">
       <c r="A111" s="5" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B111" s="7">
         <v>750633919</v>
       </c>
       <c r="C111" s="29" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D111" s="32" t="s">
         <v>17</v>
@@ -4524,13 +4524,13 @@
     </row>
     <row r="112" spans="1:4" ht="15.75">
       <c r="A112" s="5" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B112" s="7">
         <v>748663895</v>
       </c>
       <c r="C112" s="29" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D112" s="32" t="s">
         <v>44</v>
@@ -4538,13 +4538,13 @@
     </row>
     <row r="113" spans="1:4" ht="15.75">
       <c r="A113" s="5" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B113" s="7">
         <v>757025119</v>
       </c>
       <c r="C113" s="29" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="D113" s="32" t="s">
         <v>17</v>
@@ -4552,13 +4552,13 @@
     </row>
     <row r="114" spans="1:4" ht="15.75">
       <c r="A114" s="5" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B114" s="7">
         <v>754842409</v>
       </c>
       <c r="C114" s="29" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D114" s="32" t="s">
         <v>17</v>
@@ -4566,13 +4566,13 @@
     </row>
     <row r="115" spans="1:4" ht="15.75">
       <c r="A115" s="5" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B115" s="7">
         <v>750634339</v>
       </c>
       <c r="C115" s="29" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="D115" s="32" t="s">
         <v>17</v>
@@ -4580,13 +4580,13 @@
     </row>
     <row r="116" spans="1:4" ht="15.75">
       <c r="A116" s="5" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B116" s="7">
         <v>748663747</v>
       </c>
       <c r="C116" s="29" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="D116" s="32" t="s">
         <v>44</v>
@@ -4594,13 +4594,13 @@
     </row>
     <row r="117" spans="1:4" ht="15.75">
       <c r="A117" s="5" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B117" s="7">
         <v>748664539</v>
       </c>
       <c r="C117" s="29" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="D117" s="32" t="s">
         <v>44</v>
@@ -4608,13 +4608,13 @@
     </row>
     <row r="118" spans="1:4" ht="15.75">
       <c r="A118" s="5" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B118" s="7">
         <v>748664943</v>
       </c>
       <c r="C118" s="29" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="D118" s="32" t="s">
         <v>44</v>
@@ -4622,13 +4622,13 @@
     </row>
     <row r="119" spans="1:4" ht="15.75">
       <c r="A119" s="5" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B119" s="7">
         <v>748663812</v>
       </c>
       <c r="C119" s="29" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D119" s="32" t="s">
         <v>44</v>
@@ -4636,13 +4636,13 @@
     </row>
     <row r="120" spans="1:4" ht="15.75">
       <c r="A120" s="5" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B120" s="7">
         <v>748664455</v>
       </c>
       <c r="C120" s="29" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D120" s="32" t="s">
         <v>17</v>
@@ -4650,13 +4650,13 @@
     </row>
     <row r="121" spans="1:4" ht="15.75">
       <c r="A121" s="5" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B121" s="7">
         <v>748664968</v>
       </c>
       <c r="C121" s="29" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D121" s="32" t="s">
         <v>44</v>
@@ -4664,13 +4664,13 @@
     </row>
     <row r="122" spans="1:4" ht="15.75">
       <c r="A122" s="5" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B122" s="7">
         <v>748664950</v>
       </c>
       <c r="C122" s="29" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D122" s="32" t="s">
         <v>17</v>
@@ -4678,13 +4678,13 @@
     </row>
     <row r="123" spans="1:4" ht="15.75">
       <c r="A123" s="5" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B123" s="7">
         <v>746942713</v>
       </c>
       <c r="C123" s="29" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D123" s="32" t="s">
         <v>44</v>
@@ -4692,13 +4692,13 @@
     </row>
     <row r="124" spans="1:4" ht="15.75">
       <c r="A124" s="5" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B124" s="7">
         <v>748664984</v>
       </c>
       <c r="C124" s="29" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D124" s="32" t="s">
         <v>44</v>
@@ -4706,13 +4706,13 @@
     </row>
     <row r="125" spans="1:4" ht="15.75">
       <c r="A125" s="5" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B125" s="7">
         <v>752388223</v>
       </c>
       <c r="C125" s="29" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="D125" s="32" t="s">
         <v>44</v>
@@ -4720,25 +4720,25 @@
     </row>
     <row r="126" spans="1:4" ht="15.75">
       <c r="A126" s="5" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B126" s="7">
         <v>752388256</v>
       </c>
       <c r="C126" s="29" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="D126" s="25"/>
     </row>
     <row r="127" spans="1:4" ht="15.75">
       <c r="A127" s="5" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B127" s="7">
         <v>752388249</v>
       </c>
       <c r="C127" s="29" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D127" s="32" t="s">
         <v>44</v>
@@ -4746,13 +4746,13 @@
     </row>
     <row r="128" spans="1:4" ht="15.75">
       <c r="A128" s="5" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B128" s="7">
         <v>752388231</v>
       </c>
       <c r="C128" s="29" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="D128" s="32" t="s">
         <v>44</v>
@@ -4760,13 +4760,13 @@
     </row>
     <row r="129" spans="1:4" ht="15.75">
       <c r="A129" s="5" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B129" s="7">
         <v>752388264</v>
       </c>
       <c r="C129" s="29" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D129" s="32" t="s">
         <v>17</v>
@@ -4774,13 +4774,13 @@
     </row>
     <row r="130" spans="1:4" ht="15.75">
       <c r="A130" s="5" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B130" s="7">
         <v>752388306</v>
       </c>
       <c r="C130" s="29" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="D130" s="32" t="s">
         <v>44</v>
@@ -4788,13 +4788,13 @@
     </row>
     <row r="131" spans="1:4" ht="15.75">
       <c r="A131" s="5" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="B131" s="7">
         <v>752388314</v>
       </c>
       <c r="C131" s="29" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="D131" s="32" t="s">
         <v>17</v>
@@ -4802,13 +4802,13 @@
     </row>
     <row r="132" spans="1:4" ht="15.75">
       <c r="A132" s="5" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="B132" s="7">
         <v>748663341</v>
       </c>
       <c r="C132" s="29" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D132" s="32" t="s">
         <v>17</v>
@@ -4816,13 +4816,13 @@
     </row>
     <row r="133" spans="1:4" ht="15.75">
       <c r="A133" s="5" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B133" s="7">
         <v>752388322</v>
       </c>
       <c r="C133" s="29" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D133" s="32" t="s">
         <v>17</v>
@@ -4830,11 +4830,11 @@
     </row>
     <row r="134" spans="1:4" ht="15.75">
       <c r="A134" s="5" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B134" s="7"/>
       <c r="C134" s="29" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="D134" s="32" t="s">
         <v>17</v>
@@ -4842,13 +4842,13 @@
     </row>
     <row r="135" spans="1:4" ht="15.75">
       <c r="A135" s="5" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B135" s="7">
         <v>745823345</v>
       </c>
       <c r="C135" s="29" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D135" s="32" t="s">
         <v>17</v>
@@ -4856,13 +4856,13 @@
     </row>
     <row r="136" spans="1:4" ht="15.75">
       <c r="A136" s="5" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B136" s="7">
         <v>752390419</v>
       </c>
       <c r="C136" s="29" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="D136" s="32" t="s">
         <v>44</v>
@@ -4870,13 +4870,13 @@
     </row>
     <row r="137" spans="1:4" ht="15.75">
       <c r="A137" s="5" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B137" s="7">
         <v>752388330</v>
       </c>
       <c r="C137" s="29" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D137" s="32" t="s">
         <v>44</v>
@@ -4884,13 +4884,13 @@
     </row>
     <row r="138" spans="1:4" ht="15.75">
       <c r="A138" s="5" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B138" s="7">
         <v>746942777</v>
       </c>
       <c r="C138" s="29" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="D138" s="32" t="s">
         <v>44</v>
@@ -4898,25 +4898,25 @@
     </row>
     <row r="139" spans="1:4" ht="15.75">
       <c r="A139" s="5" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B139" s="7">
         <v>752388355</v>
       </c>
       <c r="C139" s="29" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="D139" s="25"/>
     </row>
     <row r="140" spans="1:4" ht="15.75">
       <c r="A140" s="5" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B140" s="7">
         <v>752390351</v>
       </c>
       <c r="C140" s="29" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="D140" s="32" t="s">
         <v>17</v>
@@ -4924,13 +4924,13 @@
     </row>
     <row r="141" spans="1:4" ht="15.75">
       <c r="A141" s="5" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B141" s="7">
         <v>752390393</v>
       </c>
       <c r="C141" s="29" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="D141" s="32" t="s">
         <v>44</v>
@@ -4938,13 +4938,13 @@
     </row>
     <row r="142" spans="1:4" ht="15.75">
       <c r="A142" s="5" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B142" s="7">
         <v>748663846</v>
       </c>
       <c r="C142" s="29" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="D142" s="32" t="s">
         <v>17</v>
@@ -4952,13 +4952,13 @@
     </row>
     <row r="143" spans="1:4" ht="15.75">
       <c r="A143" s="5" t="s">
-        <v>16</v>
+        <v>305</v>
       </c>
       <c r="B143" s="7">
         <v>756133740</v>
       </c>
       <c r="C143" s="29" t="s">
-        <v>15</v>
+        <v>306</v>
       </c>
       <c r="D143" s="32" t="s">
         <v>17</v>
@@ -5320,7 +5320,7 @@
         <v>756250437</v>
       </c>
       <c r="C169" s="29" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D169" s="32" t="s">
         <v>44</v>

</xml_diff>

<commit_message>
alteracao na etapa de pagamento
</commit_message>
<xml_diff>
--- a/src/bots/jmendes/excel_files/Robô Jmendes.xlsx
+++ b/src/bots/jmendes/excel_files/Robô Jmendes.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29711"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="67390" documentId="11_92485C45C1F39E42E268565A893E8C18510380CC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B456695-5CB7-49D7-AB3C-53AA9C5A9A68}"/>
+  <xr:revisionPtr revIDLastSave="67417" documentId="11_92485C45C1F39E42E268565A893E8C18510380CC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{747624E6-3509-46E9-8B15-F88EEF671078}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="393">
   <si>
     <t>Data</t>
   </si>
@@ -58,7 +58,7 @@
     <t>Gestão</t>
   </si>
   <si>
-    <t>Peso</t>
+    <t>Valor</t>
   </si>
   <si>
     <t>Natureza</t>
@@ -85,19 +85,34 @@
     <t>Situação Final</t>
   </si>
   <si>
+    <t>NJZ0571</t>
+  </si>
+  <si>
+    <t>Edinaldo Rodrigo De Almeida</t>
+  </si>
+  <si>
+    <t>Levolog</t>
+  </si>
+  <si>
+    <t>08579947000291</t>
+  </si>
+  <si>
+    <t>08689024000292</t>
+  </si>
+  <si>
     <t>MQN5475</t>
   </si>
   <si>
     <t>Antonio Dos Santos</t>
   </si>
   <si>
-    <t>Levolog</t>
-  </si>
-  <si>
-    <t>08579947000291</t>
-  </si>
-  <si>
-    <t>08689024000292</t>
+    <t>KRR7D11</t>
+  </si>
+  <si>
+    <t>Joel Martins dos Santos</t>
+  </si>
+  <si>
+    <t>FRETO LOG</t>
   </si>
   <si>
     <t>JMN</t>
@@ -956,12 +971,6 @@
     <t>HIM3822</t>
   </si>
   <si>
-    <t>Edinaldo Rodrigo De Almeida</t>
-  </si>
-  <si>
-    <t>NJZ0571</t>
-  </si>
-  <si>
     <t>Rodrigo de Oliveira</t>
   </si>
   <si>
@@ -1113,9 +1122,6 @@
   </si>
   <si>
     <t>JOEL MARTINS DOS SANTOS</t>
-  </si>
-  <si>
-    <t>KRR7D11</t>
   </si>
   <si>
     <t>MATHEUS FELIPE DIAS</t>
@@ -1218,6 +1224,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+  </numFmts>
   <fonts count="11">
     <font>
       <sz val="11"/>
@@ -1719,7 +1728,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1853,6 +1862,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2183,7 +2195,7 @@
     <col min="1" max="1" width="17.7109375" style="57" customWidth="1"/>
     <col min="2" max="2" width="17.85546875" style="1" customWidth="1"/>
     <col min="3" max="3" width="24.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="39.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="34.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19.5703125" style="1" customWidth="1"/>
     <col min="7" max="7" width="13.28515625" style="56" customWidth="1"/>
@@ -2249,13 +2261,13 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" s="62">
-        <v>46035</v>
+        <v>46037</v>
       </c>
       <c r="B2" s="1">
-        <v>637502</v>
+        <v>637983</v>
       </c>
       <c r="C2" s="1">
-        <v>754842318</v>
+        <v>756133740</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>15</v>
@@ -2266,8 +2278,8 @@
       <c r="F2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="1">
-        <v>25200</v>
+      <c r="G2" s="63">
+        <v>287.72800000000001</v>
       </c>
       <c r="H2" s="59">
         <v>97</v>
@@ -2287,28 +2299,81 @@
       <c r="M2" s="60"/>
     </row>
     <row r="3" spans="1:20">
-      <c r="A3" s="62"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="59"/>
-      <c r="L3" s="59"/>
+      <c r="A3" s="62">
+        <v>46037</v>
+      </c>
+      <c r="B3" s="1">
+        <v>638034</v>
+      </c>
+      <c r="C3" s="1">
+        <v>756133740</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="63">
+        <v>291.31200000000001</v>
+      </c>
+      <c r="H3" s="59">
+        <v>97</v>
+      </c>
+      <c r="I3" s="59">
+        <v>2797</v>
+      </c>
+      <c r="J3" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K3" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L3" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M3" s="60"/>
     </row>
     <row r="4" spans="1:20" s="50" customFormat="1">
-      <c r="A4" s="62"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="59"/>
-      <c r="I4" s="59"/>
-      <c r="J4" s="59"/>
-      <c r="K4" s="59"/>
-      <c r="L4" s="59"/>
+      <c r="A4" s="62">
+        <v>46037</v>
+      </c>
+      <c r="B4" s="1">
+        <v>638078</v>
+      </c>
+      <c r="C4" s="1">
+        <v>756133740</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="63">
+        <v>291.31200000000001</v>
+      </c>
+      <c r="H4" s="59">
+        <v>97</v>
+      </c>
+      <c r="I4" s="59">
+        <v>2797</v>
+      </c>
+      <c r="J4" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K4" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L4" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M4" s="59"/>
       <c r="N4" s="1"/>
       <c r="O4" s="59"/>
@@ -2319,18 +2384,42 @@
       <c r="T4" s="59"/>
     </row>
     <row r="5" spans="1:20" s="50" customFormat="1">
-      <c r="A5" s="62"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="59"/>
-      <c r="I5" s="59"/>
-      <c r="J5" s="59"/>
-      <c r="K5" s="59"/>
-      <c r="L5" s="59"/>
+      <c r="A5" s="62">
+        <v>46037</v>
+      </c>
+      <c r="B5" s="1">
+        <v>637936</v>
+      </c>
+      <c r="C5" s="1">
+        <v>756133740</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="63">
+        <v>288.95999999999998</v>
+      </c>
+      <c r="H5" s="59">
+        <v>97</v>
+      </c>
+      <c r="I5" s="59">
+        <v>2797</v>
+      </c>
+      <c r="J5" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K5" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L5" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M5" s="60"/>
       <c r="N5" s="49"/>
       <c r="O5" s="49"/>
@@ -2341,18 +2430,42 @@
       <c r="T5" s="49"/>
     </row>
     <row r="6" spans="1:20" s="50" customFormat="1">
-      <c r="A6" s="62"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="59"/>
-      <c r="I6" s="59"/>
-      <c r="J6" s="59"/>
-      <c r="K6" s="59"/>
-      <c r="L6" s="59"/>
+      <c r="A6" s="62">
+        <v>46037</v>
+      </c>
+      <c r="B6" s="1">
+        <v>638048</v>
+      </c>
+      <c r="C6" s="1">
+        <v>754842318</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="63">
+        <v>289.85599999999999</v>
+      </c>
+      <c r="H6" s="59">
+        <v>97</v>
+      </c>
+      <c r="I6" s="59">
+        <v>2797</v>
+      </c>
+      <c r="J6" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K6" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L6" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M6" s="60"/>
       <c r="N6" s="49"/>
       <c r="O6" s="1"/>
@@ -2363,64 +2476,238 @@
       <c r="T6"/>
     </row>
     <row r="7" spans="1:20">
-      <c r="A7" s="62"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="59"/>
-      <c r="I7" s="59"/>
-      <c r="J7" s="59"/>
-      <c r="K7" s="59"/>
-      <c r="L7" s="59"/>
+      <c r="A7" s="62">
+        <v>46037</v>
+      </c>
+      <c r="B7" s="1">
+        <v>638101</v>
+      </c>
+      <c r="C7" s="1">
+        <v>754842318</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" s="63">
+        <v>285.71199999999999</v>
+      </c>
+      <c r="H7" s="59">
+        <v>97</v>
+      </c>
+      <c r="I7" s="59">
+        <v>2797</v>
+      </c>
+      <c r="J7" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K7" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L7" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M7" s="60"/>
       <c r="N7" s="49"/>
     </row>
     <row r="8" spans="1:20">
-      <c r="A8" s="62"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="59"/>
-      <c r="I8" s="59"/>
-      <c r="J8" s="59"/>
-      <c r="K8" s="59"/>
-      <c r="L8" s="59"/>
+      <c r="A8" s="62">
+        <v>46037</v>
+      </c>
+      <c r="B8" s="1">
+        <v>638195</v>
+      </c>
+      <c r="C8" s="1">
+        <v>754842318</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="63">
+        <v>287.72800000000001</v>
+      </c>
+      <c r="H8" s="59">
+        <v>97</v>
+      </c>
+      <c r="I8" s="59">
+        <v>2797</v>
+      </c>
+      <c r="J8" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K8" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L8" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M8" s="60"/>
     </row>
     <row r="9" spans="1:20">
-      <c r="A9" s="62"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="59"/>
-      <c r="I9" s="59"/>
-      <c r="J9" s="59"/>
-      <c r="K9" s="59"/>
-      <c r="L9" s="59"/>
+      <c r="A9" s="62">
+        <v>46037</v>
+      </c>
+      <c r="B9" s="1">
+        <v>638235</v>
+      </c>
+      <c r="C9" s="1">
+        <v>754842318</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" s="63">
+        <v>285.37599999999998</v>
+      </c>
+      <c r="H9" s="59">
+        <v>97</v>
+      </c>
+      <c r="I9" s="59">
+        <v>2797</v>
+      </c>
+      <c r="J9" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K9" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L9" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M9" s="60"/>
     </row>
     <row r="10" spans="1:20">
-      <c r="A10" s="62"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="59"/>
-      <c r="I10" s="59"/>
-      <c r="J10" s="59"/>
-      <c r="K10" s="59"/>
-      <c r="L10" s="59"/>
+      <c r="A10" s="62">
+        <v>46037</v>
+      </c>
+      <c r="B10" s="1">
+        <v>638137</v>
+      </c>
+      <c r="C10" s="1">
+        <v>757316229</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G10" s="63">
+        <v>297.69599999999997</v>
+      </c>
+      <c r="H10" s="59">
+        <v>97</v>
+      </c>
+      <c r="I10" s="59">
+        <v>1989</v>
+      </c>
+      <c r="J10" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K10" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L10" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M10" s="60"/>
     </row>
     <row r="11" spans="1:20">
-      <c r="A11" s="62"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="59"/>
-      <c r="I11" s="59"/>
-      <c r="J11" s="59"/>
-      <c r="K11" s="59"/>
-      <c r="L11" s="59"/>
+      <c r="A11" s="62">
+        <v>46037</v>
+      </c>
+      <c r="B11" s="1">
+        <v>638174</v>
+      </c>
+      <c r="C11" s="1">
+        <v>757316229</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" s="63">
+        <v>294.89599999999996</v>
+      </c>
+      <c r="H11" s="59">
+        <v>97</v>
+      </c>
+      <c r="I11" s="59">
+        <v>1989</v>
+      </c>
+      <c r="J11" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K11" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L11" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M11" s="60"/>
     </row>
     <row r="12" spans="1:20">
-      <c r="A12" s="62"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="59"/>
-      <c r="I12" s="59"/>
-      <c r="J12" s="59"/>
-      <c r="K12" s="59"/>
-      <c r="L12" s="59"/>
+      <c r="A12" s="62">
+        <v>46037</v>
+      </c>
+      <c r="B12" s="1">
+        <v>638165</v>
+      </c>
+      <c r="C12" s="1">
+        <v>757316229</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G12" s="63">
+        <v>291.76</v>
+      </c>
+      <c r="H12" s="59">
+        <v>97</v>
+      </c>
+      <c r="I12" s="59">
+        <v>1989</v>
+      </c>
+      <c r="J12" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K12" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L12" s="59" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="13" spans="1:20">
       <c r="A13" s="62"/>
@@ -2834,16 +3121,16 @@
   <sheetData>
     <row r="2" spans="2:5">
       <c r="B2" s="8" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="2:5">
@@ -2851,18 +3138,18 @@
         <v>9</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="2:5">
       <c r="B4" s="11" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C4" s="1">
         <v>32.5</v>
@@ -2880,24 +3167,24 @@
         <v>18</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="2:5">
       <c r="B6" s="11" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>19</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="2:5">
@@ -2910,19 +3197,19 @@
     </row>
     <row r="9" spans="2:5">
       <c r="B9" s="17" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C9" s="18"/>
       <c r="D9" s="18" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="2:5">
       <c r="B10" s="11" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="13">
@@ -2937,18 +3224,18 @@
         <v>10</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="2:5">
       <c r="B12" s="11" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="E12" s="16"/>
     </row>
@@ -2989,18 +3276,18 @@
         <v>3</v>
       </c>
       <c r="D1" s="30" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="15.75">
       <c r="A2" s="4" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B2" s="23">
         <v>746192630</v>
       </c>
       <c r="C2" s="26" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="D2" s="32" t="s">
         <v>17</v>
@@ -3008,13 +3295,13 @@
     </row>
     <row r="3" spans="1:4" ht="15.75">
       <c r="A3" s="4" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B3" s="23">
         <v>756250122</v>
       </c>
       <c r="C3" s="26" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="D3" s="32" t="s">
         <v>17</v>
@@ -3022,13 +3309,13 @@
     </row>
     <row r="4" spans="1:4" ht="15.75">
       <c r="A4" s="4" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B4" s="23">
         <v>746942722</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="D4" s="32" t="s">
         <v>17</v>
@@ -3036,41 +3323,41 @@
     </row>
     <row r="5" spans="1:4" ht="15.75">
       <c r="A5" s="4" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B5" s="23">
         <v>746945612</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="D5" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.75">
       <c r="A6" s="4" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B6" s="23">
         <v>754842045</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D6" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.75">
       <c r="A7" s="4" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B7" s="23">
         <v>756250130</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="D7" s="32" t="s">
         <v>17</v>
@@ -3078,123 +3365,123 @@
     </row>
     <row r="8" spans="1:4" ht="15.75">
       <c r="A8" s="4" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B8" s="23">
         <v>746945676</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="D8" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.75">
       <c r="A9" s="4" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B9" s="23">
         <v>746192818</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="D9" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15.75">
       <c r="A10" s="4" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B10" s="23">
         <v>746192738</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="D10" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15.75">
       <c r="A11" s="4" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B11" s="23">
         <v>746942697</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="D11" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15.75">
       <c r="A12" s="4" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B12" s="23">
         <v>746183203</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="D12" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="15.75">
       <c r="A13" s="4" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B13" s="23"/>
       <c r="C13" s="26" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D13" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="15.75">
       <c r="A14" s="4" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="B14" s="23">
         <v>746192676</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="D14" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="15.75">
       <c r="A15" s="4" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B15" s="23">
         <v>746942811</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="D15" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="15.75">
       <c r="A16" s="4" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B16" s="23">
         <v>746192658</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="D16" s="32" t="s">
         <v>17</v>
@@ -3202,13 +3489,13 @@
     </row>
     <row r="17" spans="1:4" ht="15.75">
       <c r="A17" s="4" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="B17" s="23">
         <v>746942731</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="D17" s="32" t="s">
         <v>17</v>
@@ -3216,55 +3503,55 @@
     </row>
     <row r="18" spans="1:4" ht="15.75">
       <c r="A18" s="4" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B18" s="23">
         <v>747305019</v>
       </c>
       <c r="C18" s="26" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="D18" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="15.75">
       <c r="A19" s="4" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B19" s="23">
         <v>747303865</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="D19" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="15.75">
       <c r="A20" s="4" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B20" s="23">
         <v>746192649</v>
       </c>
       <c r="C20" s="26" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="D20" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="15.75">
       <c r="A21" s="4" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B21" s="23">
         <v>746942740</v>
       </c>
       <c r="C21" s="26" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="D21" s="32" t="s">
         <v>17</v>
@@ -3272,47 +3559,47 @@
     </row>
     <row r="22" spans="1:4" ht="15.75">
       <c r="A22" s="4" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B22" s="23">
         <v>746192783</v>
       </c>
       <c r="C22" s="26" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="D22" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="15.75">
       <c r="A23" s="4" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="B23" s="23">
         <v>754747632</v>
       </c>
       <c r="C23" s="26" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D23" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="15.75">
       <c r="A24" s="4" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B24" s="23">
         <v>746945505</v>
       </c>
       <c r="C24" s="26"/>
       <c r="D24" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="15.75">
       <c r="A25" s="4" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B25" s="23">
         <v>747305050</v>
@@ -3322,13 +3609,13 @@
     </row>
     <row r="26" spans="1:4" ht="15.75">
       <c r="A26" s="4" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B26" s="23">
         <v>746192774</v>
       </c>
       <c r="C26" s="26" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="D26" s="32" t="s">
         <v>17</v>
@@ -3336,13 +3623,13 @@
     </row>
     <row r="27" spans="1:4" ht="15.75">
       <c r="A27" s="4" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="B27" s="23">
         <v>744145848</v>
       </c>
       <c r="C27" s="26" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="D27" s="32" t="s">
         <v>17</v>
@@ -3350,13 +3637,13 @@
     </row>
     <row r="28" spans="1:4" ht="15.75">
       <c r="A28" s="4" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B28" s="23">
         <v>746942839</v>
       </c>
       <c r="C28" s="26" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D28" s="32" t="s">
         <v>17</v>
@@ -3364,41 +3651,41 @@
     </row>
     <row r="29" spans="1:4" ht="15.75">
       <c r="A29" s="4" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B29" s="23">
         <v>746192916</v>
       </c>
       <c r="C29" s="26" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D29" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="15.75">
       <c r="A30" s="4" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B30" s="23">
         <v>756250403</v>
       </c>
       <c r="C30" s="26" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D30" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="4" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="B31" s="1">
         <v>756250106</v>
       </c>
       <c r="C31" s="26" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="D31" s="32" t="s">
         <v>17</v>
@@ -3406,55 +3693,55 @@
     </row>
     <row r="32" spans="1:4" ht="15.75">
       <c r="A32" s="4" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="B32" s="23">
         <v>752388348</v>
       </c>
       <c r="C32" s="26" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="D32" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="15.75">
       <c r="A33" s="4" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B33" s="23">
         <v>748664927</v>
       </c>
       <c r="C33" s="26" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="D33" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="15.75">
       <c r="A34" s="4" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B34" s="23">
         <v>746945514</v>
       </c>
       <c r="C34" s="26" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="D34" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="15.75">
       <c r="A35" s="4" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="B35" s="23">
         <v>754842417</v>
       </c>
       <c r="C35" s="26" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D35" s="32" t="s">
         <v>17</v>
@@ -3462,55 +3749,55 @@
     </row>
     <row r="36" spans="1:4" ht="15.75">
       <c r="A36" s="4" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="B36" s="23">
         <v>746183196</v>
       </c>
       <c r="C36" s="26" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="D36" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="15.75">
       <c r="A37" s="4" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B37" s="23">
         <v>756250395</v>
       </c>
       <c r="C37" s="26" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D37" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="15.75">
       <c r="A38" s="4" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B38" s="23">
         <v>756250429</v>
       </c>
       <c r="C38" s="26" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="D38" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="15.75">
       <c r="A39" s="4" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="B39" s="23">
         <v>754842359</v>
       </c>
       <c r="C39" s="26" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="D39" s="32" t="s">
         <v>17</v>
@@ -3518,13 +3805,13 @@
     </row>
     <row r="40" spans="1:4" ht="15.75">
       <c r="A40" s="4" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B40" s="23">
         <v>748664570</v>
       </c>
       <c r="C40" s="26" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="D40" s="32" t="s">
         <v>17</v>
@@ -3532,83 +3819,83 @@
     </row>
     <row r="41" spans="1:4" ht="15.75">
       <c r="A41" s="4" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B41" s="23">
         <v>754842078</v>
       </c>
       <c r="C41" s="26" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="D41" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="15.75">
       <c r="A42" s="4" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="B42" s="23">
         <v>756250411</v>
       </c>
       <c r="C42" s="26" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="D42" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="15.75">
       <c r="A43" s="4" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B43" s="23">
         <v>745892911</v>
       </c>
       <c r="C43" s="26" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="D43" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="15.75">
       <c r="A44" s="4" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="B44" s="23">
         <v>746945532</v>
       </c>
       <c r="C44" s="26" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="D44" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="15.75">
       <c r="A45" s="4" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B45" s="23">
         <v>746945541</v>
       </c>
       <c r="C45" s="26" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="D45" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="15.75">
       <c r="A46" s="4" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="B46" s="23">
         <v>746945621</v>
       </c>
       <c r="C46" s="26" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="D46" s="32" t="s">
         <v>17</v>
@@ -3616,27 +3903,27 @@
     </row>
     <row r="47" spans="1:4" ht="15.75">
       <c r="A47" s="4" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B47" s="23">
         <v>746192667</v>
       </c>
       <c r="C47" s="26" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="D47" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="15.75">
       <c r="A48" s="4" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="B48" s="23">
         <v>748664554</v>
       </c>
       <c r="C48" s="26" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="D48" s="32" t="s">
         <v>17</v>
@@ -3644,86 +3931,86 @@
     </row>
     <row r="49" spans="1:5" ht="15.75">
       <c r="A49" s="4" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B49" s="23">
         <v>748664935</v>
       </c>
       <c r="C49" s="26" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="D49" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="15.75">
       <c r="A50" s="4" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="B50" s="23">
         <v>743757377</v>
       </c>
       <c r="C50" s="26" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="D50" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="15.75">
       <c r="A51" s="4" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="B51" s="23">
         <v>754845196</v>
       </c>
       <c r="C51" s="26" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="D51" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="15.75">
       <c r="A52" s="4" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="B52" s="23">
         <v>747303964</v>
       </c>
       <c r="C52" s="26" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="D52" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="15.75">
       <c r="A53" s="4" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="B53" s="23">
         <v>746128979</v>
       </c>
       <c r="C53" s="27" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D53" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E53" s="46" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="15.75">
       <c r="A54" s="4" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="B54" s="23">
         <v>746181107</v>
       </c>
       <c r="C54" s="26" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="D54" s="32" t="s">
         <v>17</v>
@@ -3731,13 +4018,13 @@
     </row>
     <row r="55" spans="1:5" ht="15.75">
       <c r="A55" s="4" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B55" s="23">
         <v>754842367</v>
       </c>
       <c r="C55" s="26" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="D55" s="32" t="s">
         <v>17</v>
@@ -3745,27 +4032,27 @@
     </row>
     <row r="56" spans="1:5" ht="15.75">
       <c r="A56" s="4" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="B56" s="23">
         <v>747304020</v>
       </c>
       <c r="C56" s="26" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D56" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="15.75">
       <c r="A57" s="4" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B57" s="23">
         <v>752390328</v>
       </c>
       <c r="C57" s="26" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="D57" s="32" t="s">
         <v>17</v>
@@ -3773,51 +4060,51 @@
     </row>
     <row r="58" spans="1:5" ht="15.75">
       <c r="A58" s="4" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="B58" s="24"/>
       <c r="C58" s="26" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="D58" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="15.75">
       <c r="A59" s="4" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B59" s="23">
         <v>745892760</v>
       </c>
       <c r="C59" s="26" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="D59" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="15.75">
       <c r="A60" s="4" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="B60" s="23"/>
       <c r="C60" s="26" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="D60" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="15.75">
       <c r="A61" s="4" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="B61" s="23">
         <v>746942759</v>
       </c>
       <c r="C61" s="26" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="D61" s="32" t="s">
         <v>17</v>
@@ -3825,41 +4112,41 @@
     </row>
     <row r="62" spans="1:5" ht="15.75">
       <c r="A62" s="4" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B62" s="23">
         <v>745205352</v>
       </c>
       <c r="C62" s="26" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="D62" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="15.75">
       <c r="A63" s="4" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="B63" s="23">
         <v>746942768</v>
       </c>
       <c r="C63" s="26" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="D63" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="15.75">
       <c r="A64" s="4" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="B64" s="7">
         <v>754842433</v>
       </c>
       <c r="C64" s="28" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="D64" s="32" t="s">
         <v>17</v>
@@ -3867,83 +4154,83 @@
     </row>
     <row r="65" spans="1:5" ht="15.75" customHeight="1">
       <c r="A65" s="4" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="B65" s="7">
         <v>746942820</v>
       </c>
       <c r="C65" s="28" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D65" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="15.75">
       <c r="A66" s="5" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B66" s="7">
         <v>747304046</v>
       </c>
       <c r="C66" s="29" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="D66" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="15.75">
       <c r="A67" s="5" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B67" s="7">
         <v>756250270</v>
       </c>
       <c r="C67" s="29" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="D67" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="15.75">
       <c r="A68" s="5" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="B68" s="7">
         <v>755662533</v>
       </c>
       <c r="C68" s="29" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="D68" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="15.75">
       <c r="A69" s="5" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="B69" s="7">
         <v>745892779</v>
       </c>
       <c r="C69" s="29" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D69" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="15.75">
       <c r="A70" s="5" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B70" s="7">
         <v>752390302</v>
       </c>
       <c r="C70" s="29" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="D70" s="32" t="s">
         <v>17</v>
@@ -3951,13 +4238,13 @@
     </row>
     <row r="71" spans="1:5" ht="15.75">
       <c r="A71" s="5" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="B71" s="7">
         <v>745892797</v>
       </c>
       <c r="C71" s="29" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="D71" s="32" t="s">
         <v>17</v>
@@ -3965,72 +4252,72 @@
     </row>
     <row r="72" spans="1:5" ht="15.75">
       <c r="A72" s="5" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="B72" s="7" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="C72" s="29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="D72" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="15.75">
       <c r="A73" s="5" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="B73" s="7">
         <v>747303931</v>
       </c>
       <c r="C73" s="29" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="D73" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E73" s="46" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="15.75">
       <c r="A74" s="5" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B74" s="7">
         <v>744143635</v>
       </c>
       <c r="C74" s="29" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="D74" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="15.75">
       <c r="A75" s="5" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="B75" s="7">
         <v>746945541</v>
       </c>
       <c r="C75" s="29" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="D75" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="15.75">
       <c r="A76" s="5" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="B76" s="7">
         <v>747303972</v>
       </c>
       <c r="C76" s="29" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="D76" s="32" t="s">
         <v>17</v>
@@ -4038,13 +4325,13 @@
     </row>
     <row r="77" spans="1:5" ht="15.75">
       <c r="A77" s="5" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="B77" s="7">
         <v>746192701</v>
       </c>
       <c r="C77" s="29" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="D77" s="32" t="s">
         <v>17</v>
@@ -4052,13 +4339,13 @@
     </row>
     <row r="78" spans="1:5" ht="15.75">
       <c r="A78" s="5" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="B78" s="7">
         <v>745892840</v>
       </c>
       <c r="C78" s="29" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="D78" s="32" t="s">
         <v>17</v>
@@ -4066,13 +4353,13 @@
     </row>
     <row r="79" spans="1:5" ht="15.75">
       <c r="A79" s="5" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="B79" s="7">
         <v>744145848</v>
       </c>
       <c r="C79" s="29" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="D79" s="32" t="s">
         <v>17</v>
@@ -4080,27 +4367,27 @@
     </row>
     <row r="80" spans="1:5" ht="15.75">
       <c r="A80" s="5" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="B80" s="7">
         <v>745892831</v>
       </c>
       <c r="C80" s="29" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="D80" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="81" spans="1:4" ht="15.75">
       <c r="A81" s="5" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="B81" s="7">
         <v>743757377</v>
       </c>
       <c r="C81" s="29" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="D81" s="32" t="s">
         <v>17</v>
@@ -4108,13 +4395,13 @@
     </row>
     <row r="82" spans="1:4" ht="15.75">
       <c r="A82" s="5" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="B82" s="7">
         <v>752390294</v>
       </c>
       <c r="C82" s="29" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="D82" s="32" t="s">
         <v>17</v>
@@ -4122,53 +4409,53 @@
     </row>
     <row r="83" spans="1:4" ht="15.75">
       <c r="A83" s="5" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="B83" s="7">
         <v>748173721</v>
       </c>
       <c r="C83" s="29" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="D83" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="84" spans="1:4" ht="15.75">
       <c r="A84" s="5" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="B84" s="7">
         <v>748173713</v>
       </c>
       <c r="C84" s="29" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="D84" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="85" spans="1:4" ht="15.75">
       <c r="A85" s="5" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="B85" s="7">
         <v>745892822</v>
       </c>
       <c r="C85" s="29"/>
       <c r="D85" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="86" spans="1:4" ht="15.75">
       <c r="A86" s="5" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="B86" s="7">
         <v>748663648</v>
       </c>
       <c r="C86" s="29" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="D86" s="32" t="s">
         <v>17</v>
@@ -4176,13 +4463,13 @@
     </row>
     <row r="87" spans="1:4" ht="15.75">
       <c r="A87" s="5" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="B87" s="7">
         <v>746192774</v>
       </c>
       <c r="C87" s="29" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="D87" s="32" t="s">
         <v>17</v>
@@ -4190,13 +4477,13 @@
     </row>
     <row r="88" spans="1:4" ht="15.75">
       <c r="A88" s="5" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="B88" s="7">
         <v>748663432</v>
       </c>
       <c r="C88" s="29" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="D88" s="32" t="s">
         <v>17</v>
@@ -4204,41 +4491,41 @@
     </row>
     <row r="89" spans="1:4" ht="15.75">
       <c r="A89" s="5" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="B89" s="7">
         <v>748662806</v>
       </c>
       <c r="C89" s="29" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="D89" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="90" spans="1:4" ht="15.75">
       <c r="A90" s="5" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="B90" s="7">
         <v>748663465</v>
       </c>
       <c r="C90" s="29" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="D90" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="91" spans="1:4" ht="15.75">
       <c r="A91" s="5" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B91" s="7">
         <v>754842318</v>
       </c>
       <c r="C91" s="29" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D91" s="32" t="s">
         <v>17</v>
@@ -4246,13 +4533,13 @@
     </row>
     <row r="92" spans="1:4" ht="15.75">
       <c r="A92" s="5" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B92" s="7">
         <v>748173697</v>
       </c>
       <c r="C92" s="29" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="D92" s="32" t="s">
         <v>17</v>
@@ -4260,153 +4547,153 @@
     </row>
     <row r="93" spans="1:4" ht="15.75">
       <c r="A93" s="5" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="B93" s="7">
         <v>746942875</v>
       </c>
       <c r="C93" s="29" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="D93" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="94" spans="1:4" ht="15.75">
       <c r="A94" s="5" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="B94" s="7">
         <v>748173747</v>
       </c>
       <c r="C94" s="29" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="D94" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="95" spans="1:4" ht="15.75">
       <c r="A95" s="5" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="B95" s="7">
         <v>748663903</v>
       </c>
       <c r="C95" s="29" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="D95" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="96" spans="1:4" ht="15.75">
       <c r="A96" s="5" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="B96" s="7">
         <v>748662996</v>
       </c>
       <c r="C96" s="29" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="D96" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="97" spans="1:4" ht="15.75">
       <c r="A97" s="5" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="B97" s="7">
         <v>748663911</v>
       </c>
       <c r="C97" s="29" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="D97" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="98" spans="1:4" ht="15.75">
       <c r="A98" s="5" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B98" s="7">
         <v>748663390</v>
       </c>
       <c r="C98" s="29" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="D98" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="99" spans="1:4" ht="15.75">
       <c r="A99" s="5" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B99" s="7">
         <v>748663382</v>
       </c>
       <c r="C99" s="29" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="D99" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="100" spans="1:4" ht="15.75">
       <c r="A100" s="5" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="B100" s="7">
         <v>750635237</v>
       </c>
       <c r="C100" s="29" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="D100" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="101" spans="1:4" ht="15.75">
       <c r="A101" s="5" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="B101" s="7">
         <v>748664422</v>
       </c>
       <c r="C101" s="29" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="D101" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="102" spans="1:4" ht="15.75">
       <c r="A102" s="5" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="B102" s="7">
         <v>748664430</v>
       </c>
       <c r="C102" s="29" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="D102" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="103" spans="1:4" ht="15.75">
       <c r="A103" s="5" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="B103" s="7">
         <v>748664406</v>
       </c>
       <c r="C103" s="29" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="D103" s="32" t="s">
         <v>17</v>
@@ -4414,39 +4701,39 @@
     </row>
     <row r="104" spans="1:4" ht="15.75">
       <c r="A104" s="5" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="B104" s="7">
         <v>755660156</v>
       </c>
       <c r="C104" s="29" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="D104" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="5" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="B105" s="6"/>
       <c r="C105" s="29" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D105" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="106" spans="1:4" ht="15.75">
       <c r="A106" s="5" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="B106" s="7">
         <v>746181107</v>
       </c>
       <c r="C106" s="29" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="D106" s="32" t="s">
         <v>17</v>
@@ -4454,13 +4741,13 @@
     </row>
     <row r="107" spans="1:4" ht="15.75">
       <c r="A107" s="5" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="B107" s="7">
         <v>750633877</v>
       </c>
       <c r="C107" s="29" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="D107" s="32" t="s">
         <v>17</v>
@@ -4468,13 +4755,13 @@
     </row>
     <row r="108" spans="1:4" ht="15.75">
       <c r="A108" s="5" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="B108" s="7">
         <v>750634263</v>
       </c>
       <c r="C108" s="29" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="D108" s="32" t="s">
         <v>17</v>
@@ -4482,27 +4769,27 @@
     </row>
     <row r="109" spans="1:4" ht="15.75">
       <c r="A109" s="5" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="B109" s="7">
         <v>748663820</v>
       </c>
       <c r="C109" s="29" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="D109" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="110" spans="1:4" ht="15.75">
       <c r="A110" s="5" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="B110" s="7">
         <v>748664471</v>
       </c>
       <c r="C110" s="29" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="D110" s="32" t="s">
         <v>17</v>
@@ -4510,13 +4797,13 @@
     </row>
     <row r="111" spans="1:4" ht="15.75">
       <c r="A111" s="5" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="B111" s="7">
         <v>750633919</v>
       </c>
       <c r="C111" s="29" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="D111" s="32" t="s">
         <v>17</v>
@@ -4524,27 +4811,27 @@
     </row>
     <row r="112" spans="1:4" ht="15.75">
       <c r="A112" s="5" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="B112" s="7">
         <v>748663895</v>
       </c>
       <c r="C112" s="29" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="D112" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="113" spans="1:4" ht="15.75">
       <c r="A113" s="5" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="B113" s="7">
         <v>757025119</v>
       </c>
       <c r="C113" s="29" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="D113" s="32" t="s">
         <v>17</v>
@@ -4552,13 +4839,13 @@
     </row>
     <row r="114" spans="1:4" ht="15.75">
       <c r="A114" s="5" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="B114" s="7">
         <v>754842409</v>
       </c>
       <c r="C114" s="29" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="D114" s="32" t="s">
         <v>17</v>
@@ -4566,13 +4853,13 @@
     </row>
     <row r="115" spans="1:4" ht="15.75">
       <c r="A115" s="5" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="B115" s="7">
         <v>750634339</v>
       </c>
       <c r="C115" s="29" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="D115" s="32" t="s">
         <v>17</v>
@@ -4580,69 +4867,69 @@
     </row>
     <row r="116" spans="1:4" ht="15.75">
       <c r="A116" s="5" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="B116" s="7">
         <v>748663747</v>
       </c>
       <c r="C116" s="29" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="D116" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="117" spans="1:4" ht="15.75">
       <c r="A117" s="5" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="B117" s="7">
         <v>748664539</v>
       </c>
       <c r="C117" s="29" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="D117" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="118" spans="1:4" ht="15.75">
       <c r="A118" s="5" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="B118" s="7">
         <v>748664943</v>
       </c>
       <c r="C118" s="29" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="D118" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="119" spans="1:4" ht="15.75">
       <c r="A119" s="5" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="B119" s="7">
         <v>748663812</v>
       </c>
       <c r="C119" s="29" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D119" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="120" spans="1:4" ht="15.75">
       <c r="A120" s="5" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="B120" s="7">
         <v>748664455</v>
       </c>
       <c r="C120" s="29" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="D120" s="32" t="s">
         <v>17</v>
@@ -4650,27 +4937,27 @@
     </row>
     <row r="121" spans="1:4" ht="15.75">
       <c r="A121" s="5" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="B121" s="7">
         <v>748664968</v>
       </c>
       <c r="C121" s="29" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="D121" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="122" spans="1:4" ht="15.75">
       <c r="A122" s="5" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="B122" s="7">
         <v>748664950</v>
       </c>
       <c r="C122" s="29" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="D122" s="32" t="s">
         <v>17</v>
@@ -4678,95 +4965,95 @@
     </row>
     <row r="123" spans="1:4" ht="15.75">
       <c r="A123" s="5" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="B123" s="7">
         <v>746942713</v>
       </c>
       <c r="C123" s="29" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="D123" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="124" spans="1:4" ht="15.75">
       <c r="A124" s="5" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="B124" s="7">
         <v>748664984</v>
       </c>
       <c r="C124" s="29" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="D124" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="125" spans="1:4" ht="15.75">
       <c r="A125" s="5" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="B125" s="7">
         <v>752388223</v>
       </c>
       <c r="C125" s="29" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="D125" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="126" spans="1:4" ht="15.75">
       <c r="A126" s="5" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B126" s="7">
         <v>752388256</v>
       </c>
       <c r="C126" s="29" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D126" s="25"/>
     </row>
     <row r="127" spans="1:4" ht="15.75">
       <c r="A127" s="5" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="B127" s="7">
         <v>752388249</v>
       </c>
       <c r="C127" s="29" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="D127" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="128" spans="1:4" ht="15.75">
       <c r="A128" s="5" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="B128" s="7">
         <v>752388231</v>
       </c>
       <c r="C128" s="29" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="D128" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="129" spans="1:4" ht="15.75">
       <c r="A129" s="5" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="B129" s="7">
         <v>752388264</v>
       </c>
       <c r="C129" s="29" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="D129" s="32" t="s">
         <v>17</v>
@@ -4774,27 +5061,27 @@
     </row>
     <row r="130" spans="1:4" ht="15.75">
       <c r="A130" s="5" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="B130" s="7">
         <v>752388306</v>
       </c>
       <c r="C130" s="29" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="D130" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="131" spans="1:4" ht="15.75">
       <c r="A131" s="5" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="B131" s="7">
         <v>752388314</v>
       </c>
       <c r="C131" s="29" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="D131" s="32" t="s">
         <v>17</v>
@@ -4802,13 +5089,13 @@
     </row>
     <row r="132" spans="1:4" ht="15.75">
       <c r="A132" s="5" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="B132" s="7">
         <v>748663341</v>
       </c>
       <c r="C132" s="29" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="D132" s="32" t="s">
         <v>17</v>
@@ -4816,13 +5103,13 @@
     </row>
     <row r="133" spans="1:4" ht="15.75">
       <c r="A133" s="5" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="B133" s="7">
         <v>752388322</v>
       </c>
       <c r="C133" s="29" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="D133" s="32" t="s">
         <v>17</v>
@@ -4830,11 +5117,11 @@
     </row>
     <row r="134" spans="1:4" ht="15.75">
       <c r="A134" s="5" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="B134" s="7"/>
       <c r="C134" s="29" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="D134" s="32" t="s">
         <v>17</v>
@@ -4842,13 +5129,13 @@
     </row>
     <row r="135" spans="1:4" ht="15.75">
       <c r="A135" s="5" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="B135" s="7">
         <v>745823345</v>
       </c>
       <c r="C135" s="29" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="D135" s="32" t="s">
         <v>17</v>
@@ -4856,67 +5143,67 @@
     </row>
     <row r="136" spans="1:4" ht="15.75">
       <c r="A136" s="5" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="B136" s="7">
         <v>752390419</v>
       </c>
       <c r="C136" s="29" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="D136" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="137" spans="1:4" ht="15.75">
       <c r="A137" s="5" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="B137" s="7">
         <v>752388330</v>
       </c>
       <c r="C137" s="29" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="D137" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="138" spans="1:4" ht="15.75">
       <c r="A138" s="5" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="B138" s="7">
         <v>746942777</v>
       </c>
       <c r="C138" s="29" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="D138" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="139" spans="1:4" ht="15.75">
       <c r="A139" s="5" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="B139" s="7">
         <v>752388355</v>
       </c>
       <c r="C139" s="29" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="D139" s="25"/>
     </row>
     <row r="140" spans="1:4" ht="15.75">
       <c r="A140" s="5" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="B140" s="7">
         <v>752390351</v>
       </c>
       <c r="C140" s="29" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="D140" s="32" t="s">
         <v>17</v>
@@ -4924,27 +5211,27 @@
     </row>
     <row r="141" spans="1:4" ht="15.75">
       <c r="A141" s="5" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="B141" s="7">
         <v>752390393</v>
       </c>
       <c r="C141" s="29" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="D141" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="142" spans="1:4" ht="15.75">
       <c r="A142" s="5" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="B142" s="7">
         <v>748663846</v>
       </c>
       <c r="C142" s="29" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="D142" s="32" t="s">
         <v>17</v>
@@ -4952,13 +5239,13 @@
     </row>
     <row r="143" spans="1:4" ht="15.75">
       <c r="A143" s="5" t="s">
-        <v>305</v>
+        <v>16</v>
       </c>
       <c r="B143" s="7">
         <v>756133740</v>
       </c>
       <c r="C143" s="29" t="s">
-        <v>306</v>
+        <v>15</v>
       </c>
       <c r="D143" s="32" t="s">
         <v>17</v>
@@ -4966,55 +5253,55 @@
     </row>
     <row r="144" spans="1:4" ht="15.75">
       <c r="A144" s="5" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B144" s="7">
         <v>752390336</v>
       </c>
       <c r="C144" s="29" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="D144" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="145" spans="1:4" ht="15.75">
       <c r="A145" s="5" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B145" s="7">
         <v>748663853</v>
       </c>
       <c r="C145" s="29" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D145" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="146" spans="1:4" ht="15.75">
       <c r="A146" s="5" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B146" s="7">
         <v>757522479</v>
       </c>
       <c r="C146" s="29" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="D146" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="147" spans="1:4" ht="15.75">
       <c r="A147" s="5" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B147" s="7">
         <v>748663887</v>
       </c>
       <c r="C147" s="29" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="D147" s="32" t="s">
         <v>17</v>
@@ -5022,27 +5309,27 @@
     </row>
     <row r="148" spans="1:4" ht="15.75">
       <c r="A148" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B148" s="7">
         <v>752390401</v>
       </c>
       <c r="C148" s="29" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="D148" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="149" spans="1:4" ht="15.75">
       <c r="A149" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B149" s="7">
         <v>754842326</v>
       </c>
       <c r="C149" s="29" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="D149" s="32" t="s">
         <v>17</v>
@@ -5050,13 +5337,13 @@
     </row>
     <row r="150" spans="1:4" ht="15.75">
       <c r="A150" s="5" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B150" s="7">
         <v>748173762</v>
       </c>
       <c r="C150" s="29" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="D150" s="32" t="s">
         <v>17</v>
@@ -5064,13 +5351,13 @@
     </row>
     <row r="151" spans="1:4" ht="15.75">
       <c r="A151" s="5" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B151" s="7">
         <v>752390252</v>
       </c>
       <c r="C151" s="29" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="D151" s="32" t="s">
         <v>17</v>
@@ -5078,27 +5365,27 @@
     </row>
     <row r="152" spans="1:4" ht="15.75">
       <c r="A152" s="5" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B152" s="7">
         <v>752390260</v>
       </c>
       <c r="C152" s="29" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="D152" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="153" spans="1:4" ht="15.75">
       <c r="A153" s="5" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B153" s="7">
         <v>748663754</v>
       </c>
       <c r="C153" s="29" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="D153" s="32" t="s">
         <v>17</v>
@@ -5106,13 +5393,13 @@
     </row>
     <row r="154" spans="1:4" ht="15.75">
       <c r="A154" s="5" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="B154" s="7">
         <v>754842334</v>
       </c>
       <c r="C154" s="29" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="D154" s="32" t="s">
         <v>17</v>
@@ -5120,13 +5407,13 @@
     </row>
     <row r="155" spans="1:4" ht="15.75">
       <c r="A155" s="5" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B155" s="7">
         <v>748663663</v>
       </c>
       <c r="C155" s="29" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="D155" s="32" t="s">
         <v>17</v>
@@ -5134,49 +5421,49 @@
     </row>
     <row r="156" spans="1:4" ht="15.75">
       <c r="A156" s="5" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="B156" s="7">
         <v>754845089</v>
       </c>
       <c r="C156" s="29" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="D156" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="157" spans="1:4" ht="15.75">
       <c r="A157" s="5" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B157" s="7">
         <v>754803260</v>
       </c>
       <c r="C157" s="29" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="D157" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="158" spans="1:4" ht="15.75">
       <c r="A158" s="5" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="B158" s="7">
         <v>748663432</v>
       </c>
       <c r="C158" s="29" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="D158" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="159" spans="1:4" ht="15.75">
       <c r="A159" s="5" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="B159" s="7">
         <v>754845055</v>
@@ -5188,69 +5475,69 @@
     </row>
     <row r="160" spans="1:4" ht="15.75">
       <c r="A160" s="5" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B160" s="7">
         <v>754845147</v>
       </c>
       <c r="C160" s="29" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="D160" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="161" spans="1:4" ht="15.75">
       <c r="A161" s="5" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B161" s="7">
         <v>754842342</v>
       </c>
       <c r="C161" s="29" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="D161" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="162" spans="1:4" ht="15.75">
       <c r="A162" s="5" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B162" s="7">
         <v>754842300</v>
       </c>
       <c r="C162" s="29" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="D162" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="163" spans="1:4" ht="15.75">
       <c r="A163" s="5" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B163" s="7">
         <v>757316278</v>
       </c>
       <c r="C163" s="29" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="D163" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="164" spans="1:4" ht="15.75">
       <c r="A164" s="5" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B164" s="7">
         <v>755660149</v>
       </c>
       <c r="C164" s="29" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="D164" s="32" t="s">
         <v>17</v>
@@ -5258,13 +5545,13 @@
     </row>
     <row r="165" spans="1:4" ht="15.75">
       <c r="A165" s="5" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="B165" s="7">
         <v>756250114</v>
       </c>
       <c r="C165" s="29" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="D165" s="32" t="s">
         <v>17</v>
@@ -5272,13 +5559,13 @@
     </row>
     <row r="166" spans="1:4" ht="15.75">
       <c r="A166" s="5" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="B166" s="7">
         <v>756250148</v>
       </c>
       <c r="C166" s="29" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="D166" s="32" t="s">
         <v>17</v>
@@ -5286,83 +5573,83 @@
     </row>
     <row r="167" spans="1:4" ht="15.75">
       <c r="A167" s="5" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B167" s="7">
         <v>756249959</v>
       </c>
       <c r="C167" s="29" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="D167" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="168" spans="1:4" ht="15.75">
       <c r="A168" s="5" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B168" s="7">
         <v>756249967</v>
       </c>
       <c r="C168" s="29" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="D168" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="169" spans="1:4" ht="15.75">
       <c r="A169" s="5" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="B169" s="7">
         <v>756250437</v>
       </c>
       <c r="C169" s="29" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="D169" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="170" spans="1:4" ht="15.75">
       <c r="A170" s="5" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B170" s="7">
         <v>756250445</v>
       </c>
       <c r="C170" s="29" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="D170" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="171" spans="1:4" ht="15.75">
       <c r="A171" s="5" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B171" s="7">
         <v>756250304</v>
       </c>
       <c r="C171" s="49" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="D171" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="172" spans="1:4" ht="15.75">
       <c r="A172" s="5" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="B172" s="7">
         <v>757025119</v>
       </c>
       <c r="C172" s="29" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="D172" s="32" t="s">
         <v>17</v>
@@ -5370,13 +5657,13 @@
     </row>
     <row r="173" spans="1:4" ht="15.75">
       <c r="A173" s="5" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B173" s="7">
         <v>757025176</v>
       </c>
       <c r="C173" s="29" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="D173" s="32" t="s">
         <v>17</v>
@@ -5384,27 +5671,27 @@
     </row>
     <row r="174" spans="1:4" ht="15.75">
       <c r="A174" s="5" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B174" s="7">
         <v>757316229</v>
       </c>
       <c r="C174" s="29" t="s">
-        <v>358</v>
+        <v>22</v>
       </c>
       <c r="D174" s="32" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="175" spans="1:4" ht="15.75">
       <c r="A175" s="5" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B175" s="7">
         <v>757316245</v>
       </c>
       <c r="C175" s="29" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="D175" s="32" t="s">
         <v>17</v>
@@ -5412,13 +5699,13 @@
     </row>
     <row r="176" spans="1:4" ht="15.75">
       <c r="A176" s="5" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B176" s="7">
         <v>757522487</v>
       </c>
       <c r="C176" s="29" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="D176" s="32" t="s">
         <v>17</v>
@@ -5426,13 +5713,13 @@
     </row>
     <row r="177" spans="1:4" ht="15.75">
       <c r="A177" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B177" s="7">
         <v>757316286</v>
       </c>
       <c r="C177" s="29" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="D177" s="32" t="s">
         <v>17</v>
@@ -5528,7 +5815,7 @@
   <sheetData>
     <row r="2" spans="1:13">
       <c r="A2" s="42" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B2" s="35"/>
       <c r="C2" s="35"/>
@@ -5537,7 +5824,7 @@
       <c r="F2" s="35"/>
       <c r="G2" s="35"/>
       <c r="H2" s="51" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="I2" s="52"/>
       <c r="J2" s="52"/>
@@ -5552,40 +5839,40 @@
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="37" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B4" s="33" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C4" s="33" t="s">
+        <v>370</v>
+      </c>
+      <c r="D4" s="33" t="s">
+        <v>371</v>
+      </c>
+      <c r="E4" s="33" t="s">
+        <v>372</v>
+      </c>
+      <c r="G4" s="33" t="s">
+        <v>373</v>
+      </c>
+      <c r="H4" s="37" t="s">
         <v>368</v>
       </c>
-      <c r="D4" s="33" t="s">
+      <c r="I4" s="33" t="s">
         <v>369</v>
       </c>
-      <c r="E4" s="33" t="s">
+      <c r="J4" s="33" t="s">
         <v>370</v>
       </c>
-      <c r="G4" s="33" t="s">
+      <c r="K4" s="33" t="s">
         <v>371</v>
       </c>
-      <c r="H4" s="37" t="s">
-        <v>366</v>
-      </c>
-      <c r="I4" s="33" t="s">
-        <v>367</v>
-      </c>
-      <c r="J4" s="33" t="s">
-        <v>368</v>
-      </c>
-      <c r="K4" s="33" t="s">
-        <v>369</v>
-      </c>
       <c r="L4" s="33" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="M4" s="58" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -5595,40 +5882,40 @@
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="31" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="C6" s="32" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="D6" s="50" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="E6" s="32" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="G6" s="32" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="I6" s="32" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="J6" s="32" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="K6" s="50" t="s">
+        <v>377</v>
+      </c>
+      <c r="L6" s="32" t="s">
         <v>375</v>
       </c>
-      <c r="L6" s="32" t="s">
-        <v>373</v>
-      </c>
       <c r="M6" s="36" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -5638,41 +5925,41 @@
     </row>
     <row r="8" spans="1:13" ht="15.75">
       <c r="A8" s="43" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B8" s="44" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="C8" s="44" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="D8" s="44" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="E8" s="44" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="F8" s="44"/>
       <c r="G8" s="44" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="H8" s="43" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="I8" s="44" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="J8" s="44" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="K8" s="44" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="L8" s="44" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="M8" s="44" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -5682,40 +5969,40 @@
     </row>
     <row r="10" spans="1:13">
       <c r="A10" s="31" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B10" s="32" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="C10" s="32" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="D10" s="32" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="G10" s="32" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="H10" s="31" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="I10" s="32" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="J10" s="32" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="K10" s="32" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="L10" s="32" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="M10" s="36" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -5725,40 +6012,40 @@
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="31" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B12" s="32" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="C12" s="32" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="D12" s="32" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="G12" s="32" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="H12" s="31" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="I12" s="32" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="J12" s="32" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="K12" s="32" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="L12" s="32" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="M12" s="36" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -5768,40 +6055,40 @@
     </row>
     <row r="14" spans="1:13">
       <c r="A14" s="31" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B14" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="C14" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="D14" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="E14" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="G14" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="H14" s="31" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="I14" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="J14" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="K14" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="L14" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="M14" s="36" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -5844,7 +6131,7 @@
     </row>
     <row r="19" spans="1:13">
       <c r="A19" s="50" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="I19" s="34"/>
       <c r="J19" s="54"/>

</xml_diff>

<commit_message>
ajustes finais no processo do jmn e ajustes no belgo
</commit_message>
<xml_diff>
--- a/src/bots/jmendes/excel_files/Robô Jmendes.xlsx
+++ b/src/bots/jmendes/excel_files/Robô Jmendes.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29711"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="67417" documentId="11_92485C45C1F39E42E268565A893E8C18510380CC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{747624E6-3509-46E9-8B15-F88EEF671078}"/>
+  <xr:revisionPtr revIDLastSave="67443" documentId="11_92485C45C1F39E42E268565A893E8C18510380CC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F27505FA-20C5-4BC6-9499-240A41884270}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -100,19 +100,19 @@
     <t>08689024000292</t>
   </si>
   <si>
+    <t>KRR7D11</t>
+  </si>
+  <si>
+    <t>Joel Martins dos Santos</t>
+  </si>
+  <si>
+    <t>FRETO LOG</t>
+  </si>
+  <si>
     <t>MQN5475</t>
   </si>
   <si>
     <t>Antonio Dos Santos</t>
-  </si>
-  <si>
-    <t>KRR7D11</t>
-  </si>
-  <si>
-    <t>Joel Martins dos Santos</t>
-  </si>
-  <si>
-    <t>FRETO LOG</t>
   </si>
   <si>
     <t>JMN</t>
@@ -2261,10 +2261,10 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" s="62">
-        <v>46037</v>
+        <v>46038</v>
       </c>
       <c r="B2" s="1">
-        <v>637983</v>
+        <v>638230</v>
       </c>
       <c r="C2" s="1">
         <v>756133740</v>
@@ -2279,7 +2279,7 @@
         <v>17</v>
       </c>
       <c r="G2" s="63">
-        <v>287.72800000000001</v>
+        <v>292.99199999999996</v>
       </c>
       <c r="H2" s="59">
         <v>97</v>
@@ -2300,10 +2300,10 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3" s="62">
-        <v>46037</v>
+        <v>46038</v>
       </c>
       <c r="B3" s="1">
-        <v>638034</v>
+        <v>638275</v>
       </c>
       <c r="C3" s="1">
         <v>756133740</v>
@@ -2318,7 +2318,7 @@
         <v>17</v>
       </c>
       <c r="G3" s="63">
-        <v>291.31200000000001</v>
+        <v>292.65599999999995</v>
       </c>
       <c r="H3" s="59">
         <v>97</v>
@@ -2339,10 +2339,10 @@
     </row>
     <row r="4" spans="1:20" s="50" customFormat="1">
       <c r="A4" s="62">
-        <v>46037</v>
+        <v>46038</v>
       </c>
       <c r="B4" s="1">
-        <v>638078</v>
+        <v>638319</v>
       </c>
       <c r="C4" s="1">
         <v>756133740</v>
@@ -2357,7 +2357,7 @@
         <v>17</v>
       </c>
       <c r="G4" s="63">
-        <v>291.31200000000001</v>
+        <v>287.50400000000002</v>
       </c>
       <c r="H4" s="59">
         <v>97</v>
@@ -2385,10 +2385,10 @@
     </row>
     <row r="5" spans="1:20" s="50" customFormat="1">
       <c r="A5" s="62">
-        <v>46037</v>
+        <v>46038</v>
       </c>
       <c r="B5" s="1">
-        <v>637936</v>
+        <v>638353</v>
       </c>
       <c r="C5" s="1">
         <v>756133740</v>
@@ -2403,7 +2403,7 @@
         <v>17</v>
       </c>
       <c r="G5" s="63">
-        <v>288.95999999999998</v>
+        <v>294.22399999999999</v>
       </c>
       <c r="H5" s="59">
         <v>97</v>
@@ -2431,13 +2431,13 @@
     </row>
     <row r="6" spans="1:20" s="50" customFormat="1">
       <c r="A6" s="62">
-        <v>46037</v>
+        <v>46038</v>
       </c>
       <c r="B6" s="1">
-        <v>638048</v>
+        <v>638416</v>
       </c>
       <c r="C6" s="1">
-        <v>754842318</v>
+        <v>757316229</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>20</v>
@@ -2446,16 +2446,16 @@
         <v>21</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="G6" s="63">
-        <v>289.85599999999999</v>
+        <v>292.65599999999995</v>
       </c>
       <c r="H6" s="59">
         <v>97</v>
       </c>
       <c r="I6" s="59">
-        <v>2797</v>
+        <v>1989</v>
       </c>
       <c r="J6" s="59">
         <v>22666</v>
@@ -2477,13 +2477,13 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" s="62">
-        <v>46037</v>
+        <v>46038</v>
       </c>
       <c r="B7" s="1">
-        <v>638101</v>
+        <v>638366</v>
       </c>
       <c r="C7" s="1">
-        <v>754842318</v>
+        <v>757316229</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>20</v>
@@ -2492,16 +2492,16 @@
         <v>21</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="G7" s="63">
-        <v>285.71199999999999</v>
+        <v>296.46399999999994</v>
       </c>
       <c r="H7" s="59">
         <v>97</v>
       </c>
       <c r="I7" s="59">
-        <v>2797</v>
+        <v>1989</v>
       </c>
       <c r="J7" s="59">
         <v>22666</v>
@@ -2517,13 +2517,13 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" s="62">
-        <v>46037</v>
+        <v>46038</v>
       </c>
       <c r="B8" s="1">
-        <v>638195</v>
+        <v>638441</v>
       </c>
       <c r="C8" s="1">
-        <v>754842318</v>
+        <v>757316229</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>20</v>
@@ -2532,16 +2532,16 @@
         <v>21</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="G8" s="63">
-        <v>287.72800000000001</v>
+        <v>297.584</v>
       </c>
       <c r="H8" s="59">
         <v>97</v>
       </c>
       <c r="I8" s="59">
-        <v>2797</v>
+        <v>1989</v>
       </c>
       <c r="J8" s="59">
         <v>22666</v>
@@ -2556,25 +2556,25 @@
     </row>
     <row r="9" spans="1:20">
       <c r="A9" s="62">
-        <v>46037</v>
+        <v>46038</v>
       </c>
       <c r="B9" s="1">
-        <v>638235</v>
+        <v>638510</v>
       </c>
       <c r="C9" s="1">
         <v>754842318</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G9" s="63">
-        <v>285.37599999999998</v>
+        <v>288.95999999999998</v>
       </c>
       <c r="H9" s="59">
         <v>97</v>
@@ -2595,31 +2595,31 @@
     </row>
     <row r="10" spans="1:20">
       <c r="A10" s="62">
-        <v>46037</v>
+        <v>46038</v>
       </c>
       <c r="B10" s="1">
-        <v>638137</v>
+        <v>638322</v>
       </c>
       <c r="C10" s="1">
-        <v>757316229</v>
+        <v>754842318</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="G10" s="63">
-        <v>297.69599999999997</v>
+        <v>284.928</v>
       </c>
       <c r="H10" s="59">
         <v>97</v>
       </c>
       <c r="I10" s="59">
-        <v>1989</v>
+        <v>2797</v>
       </c>
       <c r="J10" s="59">
         <v>22666</v>
@@ -2634,31 +2634,31 @@
     </row>
     <row r="11" spans="1:20">
       <c r="A11" s="62">
-        <v>46037</v>
+        <v>46038</v>
       </c>
       <c r="B11" s="1">
-        <v>638174</v>
+        <v>638282</v>
       </c>
       <c r="C11" s="1">
-        <v>757316229</v>
+        <v>754842318</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="G11" s="63">
-        <v>294.89599999999996</v>
+        <v>288.28799999999995</v>
       </c>
       <c r="H11" s="59">
         <v>97</v>
       </c>
       <c r="I11" s="59">
-        <v>1989</v>
+        <v>2797</v>
       </c>
       <c r="J11" s="59">
         <v>22666</v>
@@ -2673,31 +2673,31 @@
     </row>
     <row r="12" spans="1:20">
       <c r="A12" s="62">
-        <v>46037</v>
+        <v>46038</v>
       </c>
       <c r="B12" s="1">
-        <v>638165</v>
+        <v>638561</v>
       </c>
       <c r="C12" s="1">
-        <v>757316229</v>
+        <v>754842318</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="G12" s="63">
-        <v>291.76</v>
+        <v>288.62399999999997</v>
       </c>
       <c r="H12" s="59">
         <v>97</v>
       </c>
       <c r="I12" s="59">
-        <v>1989</v>
+        <v>2797</v>
       </c>
       <c r="J12" s="59">
         <v>22666</v>
@@ -4519,13 +4519,13 @@
     </row>
     <row r="91" spans="1:4" ht="15.75">
       <c r="A91" s="5" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B91" s="7">
         <v>754842318</v>
       </c>
       <c r="C91" s="29" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D91" s="32" t="s">
         <v>17</v>
@@ -5677,7 +5677,7 @@
         <v>757316229</v>
       </c>
       <c r="C174" s="29" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D174" s="32" t="s">
         <v>49</v>

</xml_diff>

<commit_message>
ajuste no start dos bots
</commit_message>
<xml_diff>
--- a/src/bots/jmendes/excel_files/Robô Jmendes.xlsx
+++ b/src/bots/jmendes/excel_files/Robô Jmendes.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29721"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="67611" documentId="11_92485C45C1F39E42E268565A893E8C18510380CC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{681D46F4-9565-4822-9CD4-2B840DE43FC2}"/>
+  <xr:revisionPtr revIDLastSave="67706" documentId="11_92485C45C1F39E42E268565A893E8C18510380CC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB3FE076-7636-43D9-9A32-345361E0990D}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="645" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="393">
   <si>
     <t>Data</t>
   </si>
@@ -85,6 +85,39 @@
     <t>Situação Final</t>
   </si>
   <si>
+    <t>NJZ0571</t>
+  </si>
+  <si>
+    <t>Edinaldo Rodrigo de Almeida</t>
+  </si>
+  <si>
+    <t>Levolog</t>
+  </si>
+  <si>
+    <t>08579947000291</t>
+  </si>
+  <si>
+    <t>08689024000292</t>
+  </si>
+  <si>
+    <t>MQN5475</t>
+  </si>
+  <si>
+    <t>Antonio Dos Santos</t>
+  </si>
+  <si>
+    <t>Edinaldo Rodrigo De Almeida</t>
+  </si>
+  <si>
+    <t>KRR7D11</t>
+  </si>
+  <si>
+    <t>Joel Martins dos Santos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FRETO LOG </t>
+  </si>
+  <si>
     <t>JMN</t>
   </si>
   <si>
@@ -109,18 +142,12 @@
     <t>Tarifa</t>
   </si>
   <si>
-    <t>08579947000291</t>
-  </si>
-  <si>
     <t>08579947000372</t>
   </si>
   <si>
     <t>Destinatário</t>
   </si>
   <si>
-    <t>08689024000292</t>
-  </si>
-  <si>
     <t xml:space="preserve">08689024000292 </t>
   </si>
   <si>
@@ -145,9 +172,6 @@
     <t>HFD4C57</t>
   </si>
   <si>
-    <t>Levolog</t>
-  </si>
-  <si>
     <t>Rafael De Andrade</t>
   </si>
   <si>
@@ -164,9 +188,6 @@
   </si>
   <si>
     <t>QNQ5F49</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FRETO LOG </t>
   </si>
   <si>
     <t>Anderson David Reis</t>
@@ -659,12 +680,6 @@
     <t>RGB6E18</t>
   </si>
   <si>
-    <t>Antonio Dos Santos</t>
-  </si>
-  <si>
-    <t>MQN5475</t>
-  </si>
-  <si>
     <t>Milton Vieira Marciano</t>
   </si>
   <si>
@@ -956,12 +971,6 @@
     <t>HIM3822</t>
   </si>
   <si>
-    <t>Edinaldo Rodrigo De Almeida</t>
-  </si>
-  <si>
-    <t>NJZ0571</t>
-  </si>
-  <si>
     <t>Rodrigo de Oliveira</t>
   </si>
   <si>
@@ -1115,9 +1124,6 @@
     <t>JOEL MARTINS DOS SANTOS</t>
   </si>
   <si>
-    <t>KRR7D11</t>
-  </si>
-  <si>
     <t>MATHEUS FELIPE DIAS</t>
   </si>
   <si>
@@ -1208,16 +1214,10 @@
     <t>Remetente: 08579947000291</t>
   </si>
   <si>
-    <t>Remetente: '08579947000291</t>
-  </si>
-  <si>
     <t>Destinatario: 08689024000292</t>
   </si>
   <si>
     <t>Destinatario 08689024000292</t>
-  </si>
-  <si>
-    <t>Destinatario '08689024000292</t>
   </si>
 </sst>
 </file>
@@ -1728,7 +1728,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1867,6 +1867,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2260,38 +2261,120 @@
       <c r="Q1" s="49"/>
     </row>
     <row r="2" spans="1:20">
-      <c r="A2" s="62"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="59"/>
-      <c r="L2" s="59"/>
+      <c r="A2" s="62">
+        <v>46055</v>
+      </c>
+      <c r="B2" s="1">
+        <v>640647</v>
+      </c>
+      <c r="C2" s="1">
+        <v>756133740</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="1">
+        <v>292.08999999999997</v>
+      </c>
+      <c r="H2" s="59">
+        <v>97</v>
+      </c>
+      <c r="I2" s="59">
+        <v>2797</v>
+      </c>
+      <c r="J2" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K2" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L2" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M2" s="60"/>
     </row>
     <row r="3" spans="1:20">
-      <c r="A3" s="62"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="59"/>
-      <c r="L3" s="59"/>
+      <c r="A3" s="62">
+        <v>46055</v>
+      </c>
+      <c r="B3" s="1">
+        <v>640633</v>
+      </c>
+      <c r="C3" s="1">
+        <v>756133740</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="1">
+        <v>289.29000000000002</v>
+      </c>
+      <c r="H3" s="59">
+        <v>97</v>
+      </c>
+      <c r="I3" s="59">
+        <v>2797</v>
+      </c>
+      <c r="J3" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K3" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L3" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M3" s="60"/>
     </row>
     <row r="4" spans="1:20" s="50" customFormat="1">
-      <c r="A4" s="62"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="59"/>
-      <c r="I4" s="59"/>
-      <c r="J4" s="59"/>
-      <c r="K4" s="59"/>
-      <c r="L4" s="59"/>
+      <c r="A4" s="62">
+        <v>46055</v>
+      </c>
+      <c r="B4" s="1">
+        <v>640615</v>
+      </c>
+      <c r="C4" s="1">
+        <v>756133740</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="1">
+        <v>287.83999999999997</v>
+      </c>
+      <c r="H4" s="59">
+        <v>97</v>
+      </c>
+      <c r="I4" s="59">
+        <v>2797</v>
+      </c>
+      <c r="J4" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K4" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L4" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M4" s="59"/>
       <c r="N4" s="1"/>
       <c r="O4" s="59"/>
@@ -2302,18 +2385,42 @@
       <c r="T4" s="59"/>
     </row>
     <row r="5" spans="1:20" s="50" customFormat="1">
-      <c r="A5" s="62"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="59"/>
-      <c r="I5" s="59"/>
-      <c r="J5" s="59"/>
-      <c r="K5" s="59"/>
-      <c r="L5" s="59"/>
+      <c r="A5" s="62">
+        <v>46055</v>
+      </c>
+      <c r="B5" s="1">
+        <v>640899</v>
+      </c>
+      <c r="C5" s="1">
+        <v>754842318</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="1">
+        <v>285.14999999999998</v>
+      </c>
+      <c r="H5" s="59">
+        <v>97</v>
+      </c>
+      <c r="I5" s="59">
+        <v>2797</v>
+      </c>
+      <c r="J5" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K5" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L5" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M5" s="60"/>
       <c r="N5" s="49"/>
       <c r="O5" s="49"/>
@@ -2324,18 +2431,42 @@
       <c r="T5" s="49"/>
     </row>
     <row r="6" spans="1:20" s="50" customFormat="1">
-      <c r="A6" s="62"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="59"/>
-      <c r="I6" s="59"/>
-      <c r="J6" s="59"/>
-      <c r="K6" s="59"/>
-      <c r="L6" s="59"/>
+      <c r="A6" s="62">
+        <v>46055</v>
+      </c>
+      <c r="B6" s="1">
+        <v>640624</v>
+      </c>
+      <c r="C6" s="1">
+        <v>754842318</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="1">
+        <v>284.81</v>
+      </c>
+      <c r="H6" s="59">
+        <v>97</v>
+      </c>
+      <c r="I6" s="59">
+        <v>2797</v>
+      </c>
+      <c r="J6" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K6" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L6" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M6" s="60"/>
       <c r="N6" s="49"/>
       <c r="O6" s="1"/>
@@ -2346,111 +2477,431 @@
       <c r="T6"/>
     </row>
     <row r="7" spans="1:20">
-      <c r="A7" s="62"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="59"/>
-      <c r="I7" s="59"/>
-      <c r="J7" s="59"/>
-      <c r="K7" s="59"/>
-      <c r="L7" s="59"/>
+      <c r="A7" s="62">
+        <v>46055</v>
+      </c>
+      <c r="B7" s="1">
+        <v>640607</v>
+      </c>
+      <c r="C7" s="1">
+        <v>754842318</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" s="1">
+        <v>281.89999999999998</v>
+      </c>
+      <c r="H7" s="59">
+        <v>97</v>
+      </c>
+      <c r="I7" s="59">
+        <v>2797</v>
+      </c>
+      <c r="J7" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K7" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L7" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M7" s="60"/>
       <c r="N7" s="49"/>
     </row>
     <row r="8" spans="1:20">
-      <c r="A8" s="62"/>
-      <c r="H8" s="59"/>
-      <c r="I8" s="59"/>
-      <c r="J8" s="59"/>
-      <c r="K8" s="59"/>
-      <c r="L8" s="59"/>
+      <c r="A8" s="62">
+        <v>46055</v>
+      </c>
+      <c r="B8" s="1">
+        <v>640778</v>
+      </c>
+      <c r="C8" s="1">
+        <v>756133740</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="1">
+        <v>289.29000000000002</v>
+      </c>
+      <c r="H8" s="59">
+        <v>97</v>
+      </c>
+      <c r="I8" s="59">
+        <v>2797</v>
+      </c>
+      <c r="J8" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K8" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L8" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M8" s="60"/>
     </row>
     <row r="9" spans="1:20">
-      <c r="A9" s="62"/>
-      <c r="G9" s="63"/>
-      <c r="H9" s="59"/>
-      <c r="I9" s="59"/>
-      <c r="J9" s="59"/>
-      <c r="K9" s="59"/>
-      <c r="L9" s="59"/>
+      <c r="A9" s="62">
+        <v>46055</v>
+      </c>
+      <c r="B9" s="1">
+        <v>640722</v>
+      </c>
+      <c r="C9" s="1">
+        <v>756133740</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" s="1">
+        <v>293.10000000000002</v>
+      </c>
+      <c r="H9" s="59">
+        <v>97</v>
+      </c>
+      <c r="I9" s="59">
+        <v>2797</v>
+      </c>
+      <c r="J9" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K9" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L9" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M9" s="60"/>
     </row>
     <row r="10" spans="1:20">
-      <c r="A10" s="62"/>
-      <c r="G10" s="63"/>
-      <c r="H10" s="59"/>
-      <c r="I10" s="59"/>
-      <c r="J10" s="59"/>
-      <c r="K10" s="59"/>
-      <c r="L10" s="59"/>
+      <c r="A10" s="62">
+        <v>46055</v>
+      </c>
+      <c r="B10" s="1">
+        <v>640752</v>
+      </c>
+      <c r="C10" s="1">
+        <v>756133740</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G10" s="1">
+        <v>290.75</v>
+      </c>
+      <c r="H10" s="59">
+        <v>97</v>
+      </c>
+      <c r="I10" s="59">
+        <v>2797</v>
+      </c>
+      <c r="J10" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K10" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L10" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M10" s="60"/>
     </row>
     <row r="11" spans="1:20">
-      <c r="A11" s="62"/>
-      <c r="G11" s="63"/>
-      <c r="H11" s="59"/>
-      <c r="I11" s="59"/>
-      <c r="J11" s="59"/>
-      <c r="K11" s="59"/>
-      <c r="L11" s="59"/>
+      <c r="A11" s="62">
+        <v>46055</v>
+      </c>
+      <c r="B11" s="1">
+        <v>640762</v>
+      </c>
+      <c r="C11" s="1">
+        <v>756133740</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11" s="1">
+        <v>292.87999999999994</v>
+      </c>
+      <c r="H11" s="59">
+        <v>97</v>
+      </c>
+      <c r="I11" s="59">
+        <v>2797</v>
+      </c>
+      <c r="J11" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K11" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L11" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M11" s="60"/>
     </row>
     <row r="12" spans="1:20">
-      <c r="A12" s="62"/>
-      <c r="G12" s="63"/>
-      <c r="H12" s="59"/>
-      <c r="I12" s="59"/>
-      <c r="J12" s="59"/>
-      <c r="K12" s="59"/>
-      <c r="L12" s="59"/>
+      <c r="A12" s="62">
+        <v>46055</v>
+      </c>
+      <c r="B12" s="1">
+        <v>640686</v>
+      </c>
+      <c r="C12" s="1">
+        <v>757316229</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="1">
+        <v>297.69</v>
+      </c>
+      <c r="H12" s="59">
+        <v>97</v>
+      </c>
+      <c r="I12" s="59">
+        <v>1989</v>
+      </c>
+      <c r="J12" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K12" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L12" s="59" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="13" spans="1:20">
-      <c r="A13" s="62"/>
-      <c r="G13" s="63"/>
-      <c r="H13" s="59"/>
-      <c r="I13" s="59"/>
-      <c r="J13" s="59"/>
-      <c r="K13" s="59"/>
-      <c r="L13" s="59"/>
+      <c r="A13" s="62">
+        <v>46055</v>
+      </c>
+      <c r="B13" s="1">
+        <v>640679</v>
+      </c>
+      <c r="C13" s="1">
+        <v>757316229</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G13" s="1">
+        <v>298.14</v>
+      </c>
+      <c r="H13" s="59">
+        <v>97</v>
+      </c>
+      <c r="I13" s="59">
+        <v>1989</v>
+      </c>
+      <c r="J13" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K13" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L13" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="N13" s="49"/>
     </row>
     <row r="14" spans="1:20">
-      <c r="A14" s="62"/>
-      <c r="G14" s="63"/>
-      <c r="H14" s="59"/>
-      <c r="I14" s="59"/>
-      <c r="J14" s="59"/>
-      <c r="K14" s="59"/>
-      <c r="L14" s="59"/>
+      <c r="A14" s="62">
+        <v>46055</v>
+      </c>
+      <c r="B14" s="1">
+        <v>640818</v>
+      </c>
+      <c r="C14" s="1">
+        <v>757316229</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G14" s="1">
+        <v>295.79000000000002</v>
+      </c>
+      <c r="H14" s="59">
+        <v>97</v>
+      </c>
+      <c r="I14" s="59">
+        <v>1989</v>
+      </c>
+      <c r="J14" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K14" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L14" s="59" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="15" spans="1:20">
-      <c r="A15" s="62"/>
-      <c r="G15" s="63"/>
-      <c r="H15" s="59"/>
-      <c r="I15" s="59"/>
-      <c r="J15" s="59"/>
-      <c r="K15" s="59"/>
-      <c r="L15" s="59"/>
+      <c r="A15" s="62">
+        <v>46055</v>
+      </c>
+      <c r="B15" s="1">
+        <v>640831</v>
+      </c>
+      <c r="C15" s="1">
+        <v>757316229</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G15" s="1">
+        <v>298.25</v>
+      </c>
+      <c r="H15" s="59">
+        <v>97</v>
+      </c>
+      <c r="I15" s="59">
+        <v>1989</v>
+      </c>
+      <c r="J15" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K15" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L15" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M15" s="60"/>
     </row>
     <row r="16" spans="1:20">
-      <c r="A16" s="62"/>
-      <c r="G16" s="63"/>
-      <c r="H16" s="59"/>
-      <c r="I16" s="59"/>
-      <c r="J16" s="59"/>
-      <c r="K16" s="59"/>
-      <c r="L16" s="59"/>
+      <c r="A16" s="62">
+        <v>46055</v>
+      </c>
+      <c r="B16" s="1">
+        <v>640805</v>
+      </c>
+      <c r="C16" s="1">
+        <v>757316229</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G16" s="1">
+        <v>296.68</v>
+      </c>
+      <c r="H16" s="59">
+        <v>97</v>
+      </c>
+      <c r="I16" s="59">
+        <v>1989</v>
+      </c>
+      <c r="J16" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K16" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L16" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M16" s="60"/>
     </row>
     <row r="17" spans="1:20">
-      <c r="A17" s="62"/>
-      <c r="G17" s="63"/>
-      <c r="H17" s="59"/>
-      <c r="I17" s="59"/>
-      <c r="J17" s="59"/>
-      <c r="K17" s="59"/>
-      <c r="L17" s="59"/>
+      <c r="A17" s="62">
+        <v>46055</v>
+      </c>
+      <c r="B17" s="1">
+        <v>640800</v>
+      </c>
+      <c r="C17" s="1">
+        <v>757316229</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G17" s="1">
+        <v>296.35000000000002</v>
+      </c>
+      <c r="H17" s="59">
+        <v>97</v>
+      </c>
+      <c r="I17" s="59">
+        <v>1989</v>
+      </c>
+      <c r="J17" s="59">
+        <v>22666</v>
+      </c>
+      <c r="K17" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="L17" s="59" t="s">
+        <v>19</v>
+      </c>
       <c r="M17" s="60"/>
     </row>
     <row r="18" spans="1:20" s="50" customFormat="1">
@@ -2816,16 +3267,16 @@
   <sheetData>
     <row r="2" spans="2:5">
       <c r="B2" s="8" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="2:5">
@@ -2833,18 +3284,18 @@
         <v>9</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="2:5">
       <c r="B4" s="11" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="C4" s="1">
         <v>32.5</v>
@@ -2859,27 +3310,27 @@
         <v>10</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="2:5">
       <c r="B6" s="11" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="2:5">
@@ -2892,19 +3343,19 @@
     </row>
     <row r="9" spans="2:5">
       <c r="B9" s="17" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="C9" s="18"/>
       <c r="D9" s="18" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="2:5">
       <c r="B10" s="11" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="13">
@@ -2919,18 +3370,18 @@
         <v>10</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="2:5">
       <c r="B12" s="11" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="E12" s="16"/>
     </row>
@@ -2971,330 +3422,330 @@
         <v>3</v>
       </c>
       <c r="D1" s="30" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="15.75">
       <c r="A2" s="4" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="B2" s="23">
         <v>746192630</v>
       </c>
       <c r="C2" s="26" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="D2" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.75">
       <c r="A3" s="4" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B3" s="23">
         <v>756250122</v>
       </c>
       <c r="C3" s="26" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="D3" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.75">
       <c r="A4" s="4" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="B4" s="23">
         <v>746942722</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="D4" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.75">
       <c r="A5" s="4" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="B5" s="23">
         <v>746945612</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="D5" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.75">
       <c r="A6" s="4" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="B6" s="23">
         <v>754842045</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="D6" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.75">
       <c r="A7" s="4" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="B7" s="23">
         <v>756250130</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="D7" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.75">
       <c r="A8" s="4" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B8" s="23">
         <v>746945676</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="D8" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.75">
       <c r="A9" s="4" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B9" s="23">
         <v>746192818</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="D9" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15.75">
       <c r="A10" s="4" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B10" s="23">
         <v>746192738</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="D10" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15.75">
       <c r="A11" s="4" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="B11" s="23">
         <v>746942697</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="D11" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15.75">
       <c r="A12" s="4" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="B12" s="23">
         <v>746183203</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D12" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="15.75">
       <c r="A13" s="4" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B13" s="23"/>
       <c r="C13" s="26" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="D13" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="15.75">
       <c r="A14" s="4" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B14" s="23">
         <v>746192676</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="D14" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="15.75">
       <c r="A15" s="4" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="B15" s="23">
         <v>746942811</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="D15" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="15.75">
       <c r="A16" s="4" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B16" s="23">
         <v>746192658</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="D16" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15.75">
       <c r="A17" s="4" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="B17" s="23">
         <v>746942731</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="D17" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="15.75">
       <c r="A18" s="4" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="B18" s="23">
         <v>747305019</v>
       </c>
       <c r="C18" s="26" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="D18" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="15.75">
       <c r="A19" s="4" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="B19" s="23">
         <v>747303865</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="D19" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="15.75">
       <c r="A20" s="4" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="B20" s="23">
         <v>746192649</v>
       </c>
       <c r="C20" s="26" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="D20" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="15.75">
       <c r="A21" s="4" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="B21" s="23">
         <v>746942740</v>
       </c>
       <c r="C21" s="26" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="D21" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="15.75">
       <c r="A22" s="4" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B22" s="23">
         <v>746192783</v>
       </c>
       <c r="C22" s="26" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="D22" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="15.75">
       <c r="A23" s="4" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="B23" s="23">
         <v>754747632</v>
       </c>
       <c r="C23" s="26" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="D23" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="15.75">
       <c r="A24" s="4" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B24" s="23">
         <v>746945505</v>
       </c>
       <c r="C24" s="26"/>
       <c r="D24" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="15.75">
       <c r="A25" s="4" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="B25" s="23">
         <v>747305050</v>
@@ -3304,2120 +3755,2120 @@
     </row>
     <row r="26" spans="1:4" ht="15.75">
       <c r="A26" s="4" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="B26" s="23">
         <v>746192774</v>
       </c>
       <c r="C26" s="26" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="D26" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="15.75">
       <c r="A27" s="4" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="B27" s="23">
         <v>744145848</v>
       </c>
       <c r="C27" s="26" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="D27" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="15.75">
       <c r="A28" s="4" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="B28" s="23">
         <v>746942839</v>
       </c>
       <c r="C28" s="26" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="D28" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="15.75">
       <c r="A29" s="4" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="B29" s="23">
         <v>746192916</v>
       </c>
       <c r="C29" s="26" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="D29" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="15.75">
       <c r="A30" s="4" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="B30" s="23">
         <v>756250403</v>
       </c>
       <c r="C30" s="26" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="D30" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="4" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="B31" s="1">
         <v>756250106</v>
       </c>
       <c r="C31" s="26" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="D31" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="15.75">
       <c r="A32" s="4" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="B32" s="23">
         <v>752388348</v>
       </c>
       <c r="C32" s="26" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="D32" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="15.75">
       <c r="A33" s="4" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="B33" s="23">
         <v>748664927</v>
       </c>
       <c r="C33" s="26" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="D33" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="15.75">
       <c r="A34" s="4" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="B34" s="23">
         <v>746945514</v>
       </c>
       <c r="C34" s="26" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="D34" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="15.75">
       <c r="A35" s="4" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="B35" s="23">
         <v>754842417</v>
       </c>
       <c r="C35" s="26" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="D35" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="15.75">
       <c r="A36" s="4" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="B36" s="23">
         <v>746183196</v>
       </c>
       <c r="C36" s="26" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="D36" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="15.75">
       <c r="A37" s="4" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="B37" s="23">
         <v>756250395</v>
       </c>
       <c r="C37" s="26" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="D37" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="15.75">
       <c r="A38" s="4" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="B38" s="23">
         <v>756250429</v>
       </c>
       <c r="C38" s="26" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="D38" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="15.75">
       <c r="A39" s="4" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="B39" s="23">
         <v>754842359</v>
       </c>
       <c r="C39" s="26" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="D39" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="15.75">
       <c r="A40" s="4" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="B40" s="23">
         <v>748664570</v>
       </c>
       <c r="C40" s="26" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="D40" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="15.75">
       <c r="A41" s="4" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="B41" s="23">
         <v>754842078</v>
       </c>
       <c r="C41" s="26" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="D41" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="15.75">
       <c r="A42" s="4" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="B42" s="23">
         <v>756250411</v>
       </c>
       <c r="C42" s="26" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="D42" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="15.75">
       <c r="A43" s="4" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="B43" s="23">
         <v>745892911</v>
       </c>
       <c r="C43" s="26" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="D43" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="15.75">
       <c r="A44" s="4" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B44" s="23">
         <v>746945532</v>
       </c>
       <c r="C44" s="26" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="D44" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="15.75">
       <c r="A45" s="4" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="B45" s="23">
         <v>746945541</v>
       </c>
       <c r="C45" s="26" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="D45" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="15.75">
       <c r="A46" s="4" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B46" s="23">
         <v>746945621</v>
       </c>
       <c r="C46" s="26" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="D46" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="15.75">
       <c r="A47" s="4" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="B47" s="23">
         <v>746192667</v>
       </c>
       <c r="C47" s="26" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="D47" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="15.75">
       <c r="A48" s="4" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="B48" s="23">
         <v>748664554</v>
       </c>
       <c r="C48" s="26" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="D48" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="15.75">
       <c r="A49" s="4" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="B49" s="23">
         <v>748664935</v>
       </c>
       <c r="C49" s="26" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="D49" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="15.75">
       <c r="A50" s="4" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="B50" s="23">
         <v>743757377</v>
       </c>
       <c r="C50" s="26" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="D50" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="15.75">
       <c r="A51" s="4" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="B51" s="23">
         <v>754845196</v>
       </c>
       <c r="C51" s="26" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="D51" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="15.75">
       <c r="A52" s="4" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B52" s="23">
         <v>747303964</v>
       </c>
       <c r="C52" s="26" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="D52" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="15.75">
       <c r="A53" s="4" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="B53" s="23">
         <v>746128979</v>
       </c>
       <c r="C53" s="27" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="D53" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="E53" s="46" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="15.75">
       <c r="A54" s="4" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="B54" s="23">
         <v>746181107</v>
       </c>
       <c r="C54" s="26" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="D54" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="15.75">
       <c r="A55" s="4" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="B55" s="23">
         <v>754842367</v>
       </c>
       <c r="C55" s="26" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="D55" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="15.75">
       <c r="A56" s="4" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="B56" s="23">
         <v>747304020</v>
       </c>
       <c r="C56" s="26" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="D56" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="15.75">
       <c r="A57" s="4" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="B57" s="23">
         <v>752390328</v>
       </c>
       <c r="C57" s="26" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="D57" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="15.75">
       <c r="A58" s="4" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B58" s="24"/>
       <c r="C58" s="26" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="D58" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="15.75">
       <c r="A59" s="4" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B59" s="23">
         <v>745892760</v>
       </c>
       <c r="C59" s="26" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="D59" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="15.75">
       <c r="A60" s="4" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="B60" s="23"/>
       <c r="C60" s="26" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="D60" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="15.75">
       <c r="A61" s="4" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="B61" s="23">
         <v>746942759</v>
       </c>
       <c r="C61" s="26" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="D61" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="15.75">
       <c r="A62" s="4" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="B62" s="23">
         <v>745205352</v>
       </c>
       <c r="C62" s="26" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="D62" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="15.75">
       <c r="A63" s="4" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="B63" s="23">
         <v>746942768</v>
       </c>
       <c r="C63" s="26" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="D63" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="15.75">
       <c r="A64" s="4" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B64" s="7">
         <v>754842433</v>
       </c>
       <c r="C64" s="28" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="D64" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="15.75" customHeight="1">
       <c r="A65" s="4" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="B65" s="7">
         <v>746942820</v>
       </c>
       <c r="C65" s="28" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="D65" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="15.75">
       <c r="A66" s="5" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="B66" s="7">
         <v>747304046</v>
       </c>
       <c r="C66" s="29" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="D66" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="15.75">
       <c r="A67" s="5" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="B67" s="7">
         <v>756250270</v>
       </c>
       <c r="C67" s="29" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="D67" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="15.75">
       <c r="A68" s="5" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="B68" s="7">
         <v>755662533</v>
       </c>
       <c r="C68" s="29" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="D68" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="15.75">
       <c r="A69" s="5" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="B69" s="7">
         <v>745892779</v>
       </c>
       <c r="C69" s="29" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="D69" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="15.75">
       <c r="A70" s="5" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="B70" s="7">
         <v>752390302</v>
       </c>
       <c r="C70" s="29" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="D70" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="15.75">
       <c r="A71" s="5" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="B71" s="7">
         <v>745892797</v>
       </c>
       <c r="C71" s="29" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="D71" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="15.75">
       <c r="A72" s="5" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="B72" s="7" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="C72" s="29" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="D72" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="15.75">
       <c r="A73" s="5" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="B73" s="7">
         <v>747303931</v>
       </c>
       <c r="C73" s="29" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="D73" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="E73" s="46" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="15.75">
       <c r="A74" s="5" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="B74" s="7">
         <v>744143635</v>
       </c>
       <c r="C74" s="29" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="D74" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="15.75">
       <c r="A75" s="5" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="B75" s="7">
         <v>746945541</v>
       </c>
       <c r="C75" s="29" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="D75" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="15.75">
       <c r="A76" s="5" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="B76" s="7">
         <v>747303972</v>
       </c>
       <c r="C76" s="29" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="D76" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="15.75">
       <c r="A77" s="5" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="B77" s="7">
         <v>746192701</v>
       </c>
       <c r="C77" s="29" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="D77" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="15.75">
       <c r="A78" s="5" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="B78" s="7">
         <v>745892840</v>
       </c>
       <c r="C78" s="29" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="D78" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="79" spans="1:5" ht="15.75">
       <c r="A79" s="5" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="B79" s="7">
         <v>744145848</v>
       </c>
       <c r="C79" s="29" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="D79" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="80" spans="1:5" ht="15.75">
       <c r="A80" s="5" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="B80" s="7">
         <v>745892831</v>
       </c>
       <c r="C80" s="29" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="D80" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="81" spans="1:4" ht="15.75">
       <c r="A81" s="5" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="B81" s="7">
         <v>743757377</v>
       </c>
       <c r="C81" s="29" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="D81" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="82" spans="1:4" ht="15.75">
       <c r="A82" s="5" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="B82" s="7">
         <v>752390294</v>
       </c>
       <c r="C82" s="29" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="D82" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="83" spans="1:4" ht="15.75">
       <c r="A83" s="5" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="B83" s="7">
         <v>748173721</v>
       </c>
       <c r="C83" s="29" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="D83" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="84" spans="1:4" ht="15.75">
       <c r="A84" s="5" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="B84" s="7">
         <v>748173713</v>
       </c>
       <c r="C84" s="29" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="D84" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="85" spans="1:4" ht="15.75">
       <c r="A85" s="5" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="B85" s="7">
         <v>745892822</v>
       </c>
       <c r="C85" s="29"/>
       <c r="D85" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="86" spans="1:4" ht="15.75">
       <c r="A86" s="5" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="B86" s="7">
         <v>748663648</v>
       </c>
       <c r="C86" s="29" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="D86" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="87" spans="1:4" ht="15.75">
       <c r="A87" s="5" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="B87" s="7">
         <v>746192774</v>
       </c>
       <c r="C87" s="29" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="D87" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="88" spans="1:4" ht="15.75">
       <c r="A88" s="5" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="B88" s="7">
         <v>748663432</v>
       </c>
       <c r="C88" s="29" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="D88" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="89" spans="1:4" ht="15.75">
       <c r="A89" s="5" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="B89" s="7">
         <v>748662806</v>
       </c>
       <c r="C89" s="29" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="D89" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="90" spans="1:4" ht="15.75">
       <c r="A90" s="5" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="B90" s="7">
         <v>748663465</v>
       </c>
       <c r="C90" s="29" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="D90" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="91" spans="1:4" ht="15.75">
       <c r="A91" s="5" t="s">
-        <v>206</v>
+        <v>21</v>
       </c>
       <c r="B91" s="7">
         <v>754842318</v>
       </c>
       <c r="C91" s="29" t="s">
-        <v>207</v>
+        <v>20</v>
       </c>
       <c r="D91" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="15.75">
       <c r="A92" s="5" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B92" s="7">
         <v>748173697</v>
       </c>
       <c r="C92" s="29" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="D92" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="93" spans="1:4" ht="15.75">
       <c r="A93" s="5" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="B93" s="7">
         <v>746942875</v>
       </c>
       <c r="C93" s="29" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="D93" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="94" spans="1:4" ht="15.75">
       <c r="A94" s="5" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="B94" s="7">
         <v>748173747</v>
       </c>
       <c r="C94" s="29" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="D94" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="95" spans="1:4" ht="15.75">
       <c r="A95" s="5" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="B95" s="7">
         <v>748663903</v>
       </c>
       <c r="C95" s="29" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="D95" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="96" spans="1:4" ht="15.75">
       <c r="A96" s="5" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="B96" s="7">
         <v>748662996</v>
       </c>
       <c r="C96" s="29" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="D96" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="97" spans="1:4" ht="15.75">
       <c r="A97" s="5" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="B97" s="7">
         <v>748663911</v>
       </c>
       <c r="C97" s="29" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="D97" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="98" spans="1:4" ht="15.75">
       <c r="A98" s="5" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B98" s="7">
         <v>748663390</v>
       </c>
       <c r="C98" s="29" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="D98" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="99" spans="1:4" ht="15.75">
       <c r="A99" s="5" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B99" s="7">
         <v>748663382</v>
       </c>
       <c r="C99" s="29" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="D99" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="100" spans="1:4" ht="15.75">
       <c r="A100" s="5" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="B100" s="7">
         <v>750635237</v>
       </c>
       <c r="C100" s="29" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="D100" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="101" spans="1:4" ht="15.75">
       <c r="A101" s="5" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="B101" s="7">
         <v>748664422</v>
       </c>
       <c r="C101" s="29" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="D101" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="102" spans="1:4" ht="15.75">
       <c r="A102" s="5" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="B102" s="7">
         <v>748664430</v>
       </c>
       <c r="C102" s="29" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="D102" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="103" spans="1:4" ht="15.75">
       <c r="A103" s="5" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="B103" s="7">
         <v>748664406</v>
       </c>
       <c r="C103" s="29" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="D103" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="104" spans="1:4" ht="15.75">
       <c r="A104" s="5" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="B104" s="7">
         <v>755660156</v>
       </c>
       <c r="C104" s="29" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="D104" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="5" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="B105" s="6"/>
       <c r="C105" s="29" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="D105" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="106" spans="1:4" ht="15.75">
       <c r="A106" s="5" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="B106" s="7">
         <v>746181107</v>
       </c>
       <c r="C106" s="29" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="D106" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="107" spans="1:4" ht="15.75">
       <c r="A107" s="5" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="B107" s="7">
         <v>750633877</v>
       </c>
       <c r="C107" s="29" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="D107" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="108" spans="1:4" ht="15.75">
       <c r="A108" s="5" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="B108" s="7">
         <v>750634263</v>
       </c>
       <c r="C108" s="29" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="D108" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="109" spans="1:4" ht="15.75">
       <c r="A109" s="5" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="B109" s="7">
         <v>748663820</v>
       </c>
       <c r="C109" s="29" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="D109" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="110" spans="1:4" ht="15.75">
       <c r="A110" s="5" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="B110" s="7">
         <v>748664471</v>
       </c>
       <c r="C110" s="29" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="D110" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="111" spans="1:4" ht="15.75">
       <c r="A111" s="5" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="B111" s="7">
         <v>750633919</v>
       </c>
       <c r="C111" s="29" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="D111" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="112" spans="1:4" ht="15.75">
       <c r="A112" s="5" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="B112" s="7">
         <v>748663895</v>
       </c>
       <c r="C112" s="29" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="D112" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="113" spans="1:4" ht="15.75">
       <c r="A113" s="5" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="B113" s="7">
         <v>757025119</v>
       </c>
       <c r="C113" s="29" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="D113" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="114" spans="1:4" ht="15.75">
       <c r="A114" s="5" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="B114" s="7">
         <v>754842409</v>
       </c>
       <c r="C114" s="29" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="D114" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="115" spans="1:4" ht="15.75">
       <c r="A115" s="5" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="B115" s="7">
         <v>750634339</v>
       </c>
       <c r="C115" s="29" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="D115" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="116" spans="1:4" ht="15.75">
       <c r="A116" s="5" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="B116" s="7">
         <v>748663747</v>
       </c>
       <c r="C116" s="29" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="D116" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="117" spans="1:4" ht="15.75">
       <c r="A117" s="5" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="B117" s="7">
         <v>748664539</v>
       </c>
       <c r="C117" s="29" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="D117" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="118" spans="1:4" ht="15.75">
       <c r="A118" s="5" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="B118" s="7">
         <v>748664943</v>
       </c>
       <c r="C118" s="29" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="D118" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="119" spans="1:4" ht="15.75">
       <c r="A119" s="5" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="B119" s="7">
         <v>748663812</v>
       </c>
       <c r="C119" s="29" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D119" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="120" spans="1:4" ht="15.75">
       <c r="A120" s="5" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="B120" s="7">
         <v>748664455</v>
       </c>
       <c r="C120" s="29" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="D120" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="121" spans="1:4" ht="15.75">
       <c r="A121" s="5" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="B121" s="7">
         <v>748664968</v>
       </c>
       <c r="C121" s="29" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="D121" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="122" spans="1:4" ht="15.75">
       <c r="A122" s="5" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="B122" s="7">
         <v>748664950</v>
       </c>
       <c r="C122" s="29" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="D122" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="123" spans="1:4" ht="15.75">
       <c r="A123" s="5" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="B123" s="7">
         <v>746942713</v>
       </c>
       <c r="C123" s="29" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="D123" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="124" spans="1:4" ht="15.75">
       <c r="A124" s="5" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="B124" s="7">
         <v>748664984</v>
       </c>
       <c r="C124" s="29" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="D124" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="125" spans="1:4" ht="15.75">
       <c r="A125" s="5" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="B125" s="7">
         <v>752388223</v>
       </c>
       <c r="C125" s="29" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="D125" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="126" spans="1:4" ht="15.75">
       <c r="A126" s="5" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B126" s="7">
         <v>752388256</v>
       </c>
       <c r="C126" s="29" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D126" s="25"/>
     </row>
     <row r="127" spans="1:4" ht="15.75">
       <c r="A127" s="5" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="B127" s="7">
         <v>752388249</v>
       </c>
       <c r="C127" s="29" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="D127" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="128" spans="1:4" ht="15.75">
       <c r="A128" s="5" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="B128" s="7">
         <v>752388231</v>
       </c>
       <c r="C128" s="29" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="D128" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="129" spans="1:4" ht="15.75">
       <c r="A129" s="5" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="B129" s="7">
         <v>752388264</v>
       </c>
       <c r="C129" s="29" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="D129" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="130" spans="1:4" ht="15.75">
       <c r="A130" s="5" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="B130" s="7">
         <v>752388306</v>
       </c>
       <c r="C130" s="29" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="D130" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="131" spans="1:4" ht="15.75">
       <c r="A131" s="5" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="B131" s="7">
         <v>752388314</v>
       </c>
       <c r="C131" s="29" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="D131" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="132" spans="1:4" ht="15.75">
       <c r="A132" s="5" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="B132" s="7">
         <v>748663341</v>
       </c>
       <c r="C132" s="29" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="D132" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="133" spans="1:4" ht="15.75">
       <c r="A133" s="5" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="B133" s="7">
         <v>752388322</v>
       </c>
       <c r="C133" s="29" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="D133" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="134" spans="1:4" ht="15.75">
       <c r="A134" s="5" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="B134" s="7"/>
       <c r="C134" s="29" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="D134" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="135" spans="1:4" ht="15.75">
       <c r="A135" s="5" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="B135" s="7">
         <v>745823345</v>
       </c>
       <c r="C135" s="29" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="D135" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="136" spans="1:4" ht="15.75">
       <c r="A136" s="5" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="B136" s="7">
         <v>752390419</v>
       </c>
       <c r="C136" s="29" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="D136" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="137" spans="1:4" ht="15.75">
       <c r="A137" s="5" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="B137" s="7">
         <v>752388330</v>
       </c>
       <c r="C137" s="29" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="D137" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="138" spans="1:4" ht="15.75">
       <c r="A138" s="5" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="B138" s="7">
         <v>746942777</v>
       </c>
       <c r="C138" s="29" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="D138" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="139" spans="1:4" ht="15.75">
       <c r="A139" s="5" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="B139" s="7">
         <v>752388355</v>
       </c>
       <c r="C139" s="29" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="D139" s="25"/>
     </row>
     <row r="140" spans="1:4" ht="15.75">
       <c r="A140" s="5" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="B140" s="7">
         <v>752390351</v>
       </c>
       <c r="C140" s="29" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="D140" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="141" spans="1:4" ht="15.75">
       <c r="A141" s="5" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="B141" s="7">
         <v>752390393</v>
       </c>
       <c r="C141" s="29" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="D141" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="142" spans="1:4" ht="15.75">
       <c r="A142" s="5" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="B142" s="7">
         <v>748663846</v>
       </c>
       <c r="C142" s="29" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="D142" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="143" spans="1:4" ht="15.75">
       <c r="A143" s="5" t="s">
-        <v>305</v>
+        <v>22</v>
       </c>
       <c r="B143" s="7">
         <v>756133740</v>
       </c>
       <c r="C143" s="29" t="s">
-        <v>306</v>
+        <v>15</v>
       </c>
       <c r="D143" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="144" spans="1:4" ht="15.75">
       <c r="A144" s="5" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B144" s="7">
         <v>752390336</v>
       </c>
       <c r="C144" s="29" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="D144" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="145" spans="1:4" ht="15.75">
       <c r="A145" s="5" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B145" s="7">
         <v>748663853</v>
       </c>
       <c r="C145" s="29" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D145" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="146" spans="1:4" ht="15.75">
       <c r="A146" s="5" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B146" s="7">
         <v>757522479</v>
       </c>
       <c r="C146" s="29" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="D146" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="147" spans="1:4" ht="15.75">
       <c r="A147" s="5" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B147" s="7">
         <v>748663887</v>
       </c>
       <c r="C147" s="29" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="D147" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="148" spans="1:4" ht="15.75">
       <c r="A148" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B148" s="7">
         <v>752390401</v>
       </c>
       <c r="C148" s="29" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="D148" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="149" spans="1:4" ht="15.75">
       <c r="A149" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B149" s="7">
         <v>754842326</v>
       </c>
       <c r="C149" s="29" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="D149" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="150" spans="1:4" ht="15.75">
       <c r="A150" s="5" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B150" s="7">
         <v>748173762</v>
       </c>
       <c r="C150" s="29" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="D150" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="151" spans="1:4" ht="15.75">
       <c r="A151" s="5" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B151" s="7">
         <v>752390252</v>
       </c>
       <c r="C151" s="29" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="D151" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="152" spans="1:4" ht="15.75">
       <c r="A152" s="5" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B152" s="7">
         <v>752390260</v>
       </c>
       <c r="C152" s="29" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="D152" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="153" spans="1:4" ht="15.75">
       <c r="A153" s="5" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B153" s="7">
         <v>748663754</v>
       </c>
       <c r="C153" s="29" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="D153" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="154" spans="1:4" ht="15.75">
       <c r="A154" s="5" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="B154" s="7">
         <v>754842334</v>
       </c>
       <c r="C154" s="29" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="D154" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="155" spans="1:4" ht="15.75">
       <c r="A155" s="5" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B155" s="7">
         <v>748663663</v>
       </c>
       <c r="C155" s="29" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="D155" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="156" spans="1:4" ht="15.75">
       <c r="A156" s="5" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="B156" s="7">
         <v>754845089</v>
       </c>
       <c r="C156" s="29" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="D156" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="157" spans="1:4" ht="15.75">
       <c r="A157" s="5" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B157" s="7">
         <v>754803260</v>
       </c>
       <c r="C157" s="29" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="D157" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="158" spans="1:4" ht="15.75">
       <c r="A158" s="5" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="B158" s="7">
         <v>748663432</v>
       </c>
       <c r="C158" s="29" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="D158" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="159" spans="1:4" ht="15.75">
       <c r="A159" s="5" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="B159" s="7">
         <v>754845055</v>
       </c>
       <c r="C159" s="29"/>
       <c r="D159" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="160" spans="1:4" ht="15.75">
       <c r="A160" s="5" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B160" s="7">
         <v>754845147</v>
       </c>
       <c r="C160" s="29" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="D160" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="161" spans="1:4" ht="15.75">
       <c r="A161" s="5" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B161" s="7">
         <v>754842342</v>
       </c>
       <c r="C161" s="29" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="D161" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="162" spans="1:4" ht="15.75">
       <c r="A162" s="5" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="B162" s="7">
         <v>754842300</v>
       </c>
       <c r="C162" s="29" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="D162" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="163" spans="1:4" ht="15.75">
       <c r="A163" s="5" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B163" s="7">
         <v>757316278</v>
       </c>
       <c r="C163" s="29" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="D163" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="164" spans="1:4" ht="15.75">
       <c r="A164" s="5" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B164" s="7">
         <v>755660149</v>
       </c>
       <c r="C164" s="29" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="D164" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="165" spans="1:4" ht="15.75">
       <c r="A165" s="5" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="B165" s="7">
         <v>756250114</v>
       </c>
       <c r="C165" s="29" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="D165" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="166" spans="1:4" ht="15.75">
       <c r="A166" s="5" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="B166" s="7">
         <v>756250148</v>
       </c>
       <c r="C166" s="29" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="D166" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="167" spans="1:4" ht="15.75">
       <c r="A167" s="5" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B167" s="7">
         <v>756249959</v>
       </c>
       <c r="C167" s="29" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="D167" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="168" spans="1:4" ht="15.75">
       <c r="A168" s="5" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B168" s="7">
         <v>756249967</v>
       </c>
       <c r="C168" s="29" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="D168" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="169" spans="1:4" ht="15.75">
       <c r="A169" s="5" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="B169" s="7">
         <v>756250437</v>
       </c>
       <c r="C169" s="29" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="D169" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="170" spans="1:4" ht="15.75">
       <c r="A170" s="5" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B170" s="7">
         <v>756250445</v>
       </c>
       <c r="C170" s="29" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="D170" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="171" spans="1:4" ht="15.75">
       <c r="A171" s="5" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B171" s="7">
         <v>756250304</v>
       </c>
       <c r="C171" s="49" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="D171" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="172" spans="1:4" ht="15.75">
       <c r="A172" s="5" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="B172" s="7">
         <v>757025119</v>
       </c>
       <c r="C172" s="29" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="D172" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="173" spans="1:4" ht="15.75">
       <c r="A173" s="5" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B173" s="7">
         <v>757025176</v>
       </c>
       <c r="C173" s="29" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="D173" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="174" spans="1:4" ht="15.75">
       <c r="A174" s="5" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B174" s="7">
         <v>757316229</v>
       </c>
       <c r="C174" s="29" t="s">
-        <v>358</v>
+        <v>23</v>
       </c>
       <c r="D174" s="32" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="175" spans="1:4" ht="15.75">
       <c r="A175" s="5" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B175" s="7">
         <v>757316245</v>
       </c>
       <c r="C175" s="29" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="D175" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="176" spans="1:4" ht="15.75">
       <c r="A176" s="5" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B176" s="7">
         <v>757522487</v>
       </c>
       <c r="C176" s="29" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="D176" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="177" spans="1:4" ht="15.75">
       <c r="A177" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B177" s="7">
         <v>757316286</v>
       </c>
       <c r="C177" s="29" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="D177" s="32" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="178" spans="1:4" ht="15.75">
@@ -5510,7 +5961,7 @@
   <sheetData>
     <row r="2" spans="1:13">
       <c r="A2" s="42" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="B2" s="35"/>
       <c r="C2" s="35"/>
@@ -5519,7 +5970,7 @@
       <c r="F2" s="35"/>
       <c r="G2" s="35"/>
       <c r="H2" s="51" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="I2" s="52"/>
       <c r="J2" s="52"/>
@@ -5534,40 +5985,40 @@
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="37" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B4" s="33" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C4" s="33" t="s">
+        <v>370</v>
+      </c>
+      <c r="D4" s="33" t="s">
+        <v>371</v>
+      </c>
+      <c r="E4" s="33" t="s">
+        <v>372</v>
+      </c>
+      <c r="G4" s="33" t="s">
+        <v>373</v>
+      </c>
+      <c r="H4" s="37" t="s">
         <v>368</v>
       </c>
-      <c r="D4" s="33" t="s">
+      <c r="I4" s="33" t="s">
         <v>369</v>
       </c>
-      <c r="E4" s="33" t="s">
+      <c r="J4" s="33" t="s">
         <v>370</v>
       </c>
-      <c r="G4" s="33" t="s">
+      <c r="K4" s="33" t="s">
         <v>371</v>
       </c>
-      <c r="H4" s="37" t="s">
-        <v>366</v>
-      </c>
-      <c r="I4" s="33" t="s">
-        <v>367</v>
-      </c>
-      <c r="J4" s="33" t="s">
-        <v>368</v>
-      </c>
-      <c r="K4" s="33" t="s">
-        <v>369</v>
-      </c>
       <c r="L4" s="33" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="M4" s="58" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -5577,40 +6028,40 @@
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="31" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="C6" s="32" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="D6" s="50" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="E6" s="32" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="G6" s="32" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="I6" s="32" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="J6" s="32" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="K6" s="50" t="s">
+        <v>377</v>
+      </c>
+      <c r="L6" s="32" t="s">
         <v>375</v>
       </c>
-      <c r="L6" s="32" t="s">
-        <v>373</v>
-      </c>
       <c r="M6" s="36" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -5620,41 +6071,41 @@
     </row>
     <row r="8" spans="1:13" ht="15.75">
       <c r="A8" s="43" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B8" s="44" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="C8" s="44" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="D8" s="44" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="E8" s="44" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="F8" s="44"/>
       <c r="G8" s="44" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="H8" s="43" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="I8" s="44" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="J8" s="44" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="K8" s="44" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="L8" s="44" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="M8" s="44" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -5664,40 +6115,40 @@
     </row>
     <row r="10" spans="1:13">
       <c r="A10" s="31" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B10" s="32" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="C10" s="32" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="D10" s="32" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="G10" s="32" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="H10" s="31" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="I10" s="32" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="J10" s="32" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="K10" s="32" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="L10" s="32" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="M10" s="36" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -5707,40 +6158,40 @@
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="31" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B12" s="32" t="s">
-        <v>388</v>
-      </c>
-      <c r="C12" s="32" t="s">
-        <v>389</v>
+        <v>390</v>
+      </c>
+      <c r="C12" s="64" t="s">
+        <v>18</v>
       </c>
       <c r="D12" s="32" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="G12" s="32" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="H12" s="31" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="I12" s="32" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="J12" s="32" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="K12" s="32" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="L12" s="32" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="M12" s="36" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -5750,40 +6201,40 @@
     </row>
     <row r="14" spans="1:13">
       <c r="A14" s="31" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B14" s="32" t="s">
+        <v>392</v>
+      </c>
+      <c r="C14" s="64" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14" s="32" t="s">
+        <v>392</v>
+      </c>
+      <c r="E14" s="32" t="s">
+        <v>392</v>
+      </c>
+      <c r="G14" s="32" t="s">
+        <v>392</v>
+      </c>
+      <c r="H14" s="31" t="s">
         <v>391</v>
       </c>
-      <c r="C14" s="32" t="s">
+      <c r="I14" s="32" t="s">
         <v>392</v>
       </c>
-      <c r="D14" s="32" t="s">
-        <v>391</v>
-      </c>
-      <c r="E14" s="32" t="s">
-        <v>391</v>
-      </c>
-      <c r="G14" s="32" t="s">
-        <v>391</v>
-      </c>
-      <c r="H14" s="31" t="s">
-        <v>390</v>
-      </c>
-      <c r="I14" s="32" t="s">
-        <v>391</v>
-      </c>
       <c r="J14" s="32" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K14" s="32" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="L14" s="32" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="M14" s="36" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -5826,7 +6277,7 @@
     </row>
     <row r="19" spans="1:13">
       <c r="A19" s="50" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="I19" s="34"/>
       <c r="J19" s="54"/>
@@ -5834,7 +6285,7 @@
     </row>
     <row r="20" spans="1:13">
       <c r="A20" s="50" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="I20" s="34"/>
       <c r="J20" s="54"/>

</xml_diff>